<commit_message>
feat(roles): derive sourced product-manager ladder
Convert roles/product-manager from schema-migrated-but-unsourced to fully
sourced derived rendering per the normative cell-derivation rule. All 40
competencies now carry per-level bibliography sources and why-text grounded
in each capability's actual catalog P1-P6 text, plus role-specific evidence.

Hunted the known self-sourcing bug: PM-15/16/17/18/19 (7 competencies, 42
cells) were minted in 2026-07 directly from this ladder's own prior
consolidation prose, so their evidence was rewritten fresh rather than
carried over from the old ladder.md's near-identical bold clauses. Ten
anchors resolve via bibliography substitutes for citations with no entry
(Portigal, Cooper's Inmates, Olsen, McClure, Duke, Bryar & Carr, Ramanujam
& Tacke), documented in scope_note alongside the role-leveling convention
and the 13 dual-source competencies.

derived: true; ladder.md/csv/xlsx regenerated.
</commit_message>
<xml_diff>
--- a/roles/product-manager/ladder.xlsx
+++ b/roles/product-manager/ladder.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Competency Matrix" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Rating Template" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sources" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sources &amp; Theory" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -696,20 +696,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -735,35 +736,40 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Theory Anchor</t>
+          <t>What it covers</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Theory anchor &amp; why</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>P6</t>
         </is>
@@ -792,37 +798,42 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Torres, *Continuous Discovery Habits* (2021); Portigal, *Interviewing Users* (2013)</t>
+          <t>Uncovering user needs and validating problems through interviews, observation, and experimentation.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs customer interviews from a prepared story-based guide and captures verbatim notes, asking follow-up questions that pull specific past behavior rather than opinions; debriefs findings with their lead. Scope: interviews recruited for one feature or epic.</t>
+          <t>Torres, Continuous Discovery Habits: Discover Products that Create Customer Value and Business Value (Product Talk LLC, 2021) — weekly customer touchpoints with story-based, non-leading questions are the foundational discovery habit; substituted for Portigal's Interviewing Users (no bibliography entry) with fitzpatrick2013-momtest, which names the exact leading-question failure mode a script and review exist to catch.</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Maintains a weekly interviewing cadence without being told to, writing their own discussion guides, avoiding leading questions, and turning each session into snapshots teammates actually read. Scope: continuous touchpoints across their product area.</t>
+          <t>Depth: Runs scripted customer interviews and notes findings under a senior researcher's guidance. Evidenced by: Runs a scripted interview from a lead's guide, avoids the leading-question traps the Mom Test warns about, and writes up verbatim notes for the lead to review. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs the interviewing practice for their product - builds the recruiting pipeline, brings engineers and designers into sessions, and redirects interviews that drift into feature-request collection back to behavior. Scope: their product/capability; teammates cite their interview snapshots in decisions.</t>
+          <t>Depth: Plans and conducts standard discovery for a feature, synthesizing themes with normal review. Evidenced by: Keeps a weekly interview cadence going without being reminded, writes their own discussion guides, and turns each session into a snapshot teammates actually read. Scope: a product area.</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Teaches interviewing so visibly that other teams' guides and snapshot formats trace back to them; sits in on other PMs' sessions and gives technique-level feedback. Scope: interviewing practice across multiple product areas.</t>
+          <t>Depth: Independently frames ambiguous problems, selects fitting methods, and separates signal from noise. Evidenced by: Builds the recruiting pipeline for their product, brings engineers and designers into sessions, and redirects an interview that drifts into feature-request collection back to behavior. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Installs the org's interviewing infrastructure - recruiting panels, consent and incentive norms, snapshot repositories - and audits whether teams' customer contact is real or theater. Scope: product org.</t>
+          <t>Depth: Designs the team's discovery approach and untangles findings others find contradictory. Evidenced by: Reviews other PMs' discussion guides and sits in on their sessions, and the snapshot format spreading across teams traces back to their template. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the company's standard for customer contact and argues it externally in talks or writing that practitioners cite. Scope: company portfolio; executives quote customer evidence in the register this person established.</t>
+          <t>Depth: Sets the org's research strategy and anticipates emerging customer needs before they surface. Evidenced by: Stands up the org's recruiting panel, consent process, and interview-snapshot repository, and audits whether a team's customer contact is real or theater. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what rigorous product discovery means and shapes the discipline's practice externally. Evidenced by: Sets the company's public standard for what counts as real customer contact and defends it in talks or writing that other practitioners cite. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -849,37 +860,42 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Torres, *Continuous Discovery Habits* (2021); Cagan, *Inspired* (2nd ed., 2018)</t>
+          <t>Uncovering user needs and validating problems through interviews, observation, and experimentation.</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps discovery activities visible on the team board - interviews scheduled, assumptions listed, findings logged - and follows the cadence the team has set. Scope: their epic's discovery tasks.</t>
+          <t>Torres, Continuous Discovery Habits: Discover Products that Create Customer Value and Business Value (Product Talk LLC, 2021) — discovery is a weekly habit run in parallel with delivery, not a phase before it, paired with cagan2017-inspired's empowered-team framing of continuous discovery as a team default rather than a research-team hand-off.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs discovery and delivery in parallel without stalling either - the team ships weekly and talks to customers weekly, and standups show both tracks moving. Scope: the discovery rhythm of their area.</t>
+          <t>Depth: Runs scripted customer interviews and notes findings under a senior researcher's guidance. Evidenced by: Keeps their epic's discovery tasks visible on the team board — interviews scheduled, assumptions listed, findings logged — following the cadence the team already set. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sustains the discovery habit through pressure - deadlines, exec pushes, re-orgs - and visibly renegotiates scope rather than silently dropping customer contact. Scope: a product's discovery culture; their cadence is the example cited to new teams.</t>
+          <t>Depth: Plans and conducts standard discovery for a feature, synthesizing themes with normal review. Evidenced by: Runs discovery and delivery in parallel without stalling either, so standups show both a weekly ship and a weekly customer conversation moving. Scope: a product area.</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Audits discovery health across teams from artifacts and calendars, names which teams have quietly stopped learning, and gets the habit restarted. Scope: multiple product areas.</t>
+          <t>Depth: Independently frames ambiguous problems, selects fitting methods, and separates signal from noise. Evidenced by: Keeps the discovery habit alive through a deadline crunch by visibly renegotiating scope instead of quietly skipping customer contact, and new teams are pointed at their cadence as the example. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs the operating rhythm that makes discovery the default - planning rituals, review gates, and funding rules that assume continuous learning. Scope: product org.</t>
+          <t>Depth: Designs the team's discovery approach and untangles findings others find contradictory. Evidenced by: Audits discovery health across several teams from calendars and artifacts, names which team has quietly stopped learning, and gets the habit restarted. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds the company accountable to discovery at the portfolio level, challenging major investments that lack recent customer evidence in front of executive audiences. Scope: company portfolio.</t>
+          <t>Depth: Sets the org's research strategy and anticipates emerging customer needs before they surface. Evidenced by: Designs the planning rituals and funding rules that make continuous discovery the org's default rather than a practice some teams opt out of under pressure. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what rigorous product discovery means and shapes the discipline's practice externally. Evidenced by: Challenges a major company investment in an executive review for lacking recent customer evidence, and that challenge becomes the norm other reviews are held to. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -906,37 +922,42 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Torres, *Continuous Discovery Habits* (2021)</t>
+          <t>Structures discovered customer needs into an explicit opportunity space — mapped, sized, and compared — so solution choices trace to the most valuable problem rather than the first idea.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sorts interview evidence into needs, pain points, and desires on an existing opportunity map, distinguishing an opportunity from a solution when asked to label one. Scope: contributes nodes to a map their lead owns.</t>
+          <t>Torres, Continuous Discovery Habits: Discover Products that Create Customer Value and Business Value (Product Talk LLC, 2021) — the opportunity solution tree keeps teams solving customer needs rather than shipping their first idea; self-sourced capability (PM-15 was minted in 2026-07 directly from this ladder's own prior consolidation prose — see scope_note) so the evidence below is written fresh, not carried over from the old ladder.md.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds and maintains the opportunity solution tree for their area, sizing branches with evidence counts and pruning opportunities no interview supports. Scope: their product area; the tree is the artifact planning meetings open with.</t>
+          <t>Depth: Places research findings onto an existing opportunity map correctly, distinguishing opportunities from solutions with coaching. Evidenced by: Adds a newly-interviewed customer's pain point to their lead's opportunity tree in the right branch, asking when unsure whether it names a need or a disguised feature request. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Frames the target opportunity space against the product outcome and defends why one branch is being pursued over its siblings, naming the evidence and the trade-off. Scope: their product; adjacent teams borrow the map to see where their work intersects.</t>
+          <t>Depth: Builds and maintains the opportunity map for their area, sizing and pruning branches against evidence without prompting. Evidenced by: Keeps their product area's opportunity tree current between planning cycles, retiring branches no interview has touched in months and adding new ones as evidence accumulates. Scope: a product area.</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reconciles opportunity maps across teams into a shared structure, exposing duplicate bets and gaps between areas that no single team could see. Scope: multiple product areas.</t>
+          <t>Depth: Structures messy, contested problem spaces into maps that make trade-offs explicit, and defends why one opportunity is pursued over its siblings. Evidenced by: Walks a skeptical stakeholder through why the team is pursuing one opportunity over three plausible siblings, pointing at the specific interview evidence behind the call. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes opportunity mapping the org's default synthesis method, reviewing trees in strategy checkpoints and rejecting solution-first proposals that skip the structure. Scope: product org.</t>
+          <t>Depth: Reconciles overlapping opportunity maps across teams, exposing duplicate bets and orphaned opportunities no single team could see. Evidenced by: Merges two teams' opportunity trees ahead of a joint planning cycle and surfaces a customer need both teams were separately half-solving without knowing about the other's work. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes how the company represents customer needs at portfolio level, connecting opportunity structures to corporate strategy in artifacts the executive team plans against. Scope: company portfolio.</t>
+          <t>Depth: Makes opportunity mapping an organization's default synthesis method; investment reviews open from the mapped opportunity space. Evidenced by: Gets a quarterly investment review to open with the mapped opportunity space instead of a list of proposed features, and rejects a funding request that skips the map. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes how organizations represent customer opportunity at portfolio level; their framing methods are cited and reused beyond their own organization. Evidenced by: Publishes the opportunity-mapping method used across the company's product lines and fields questions about it from PMs at other companies trying to adopt it. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -963,37 +984,42 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Olsen, *The Lean Product Playbook* (2015)</t>
+          <t>Uncovering user needs and validating problems through interviews, observation, and experimentation.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Tags and clusters interview notes into themes using the team's synthesis method, and can point to the specific quotes behind each theme. Scope: synthesis for one feature's research.</t>
+          <t>Torres, Continuous Discovery Habits: Discover Products that Create Customer Value and Business Value (Product Talk LLC, 2021) — substituted for Olsen's The Lean Product Playbook (no bibliography entry) with Torres's own continuous-discovery synthesis practice — PM-01's dominant anchor — since turning raw interview notes into durable themes is the same synthesis discipline the interviewing and cadence rows above already anchor to.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Turns a batch of interviews, tickets, and usage data into a ranked set of underserved needs with the supporting evidence attached, and presents it without over-claiming. Scope: synthesis their area's decisions cite.</t>
+          <t>Depth: Runs scripted customer interviews and notes findings under a senior researcher's guidance. Evidenced by: Tags a batch of interview transcripts into the team's existing theme categories and can point to the exact quote behind each tag when a lead asks. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Integrates qualitative and quantitative evidence into insight documents that change what the team builds; peers checking their synthesis find the chain from quote to claim intact. Scope: insight base for a product; other teams cite their write-ups.</t>
+          <t>Depth: Plans and conducts standard discovery for a feature, synthesizing themes with normal review. Evidenced by: Turns three weeks of interviews and support tickets into a ranked list of underserved needs, with the evidence attached, and presents it without overclaiming. Scope: a product area.</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Spots contradictions between teams' research conclusions and forces reconciliation - same customers, conflicting claims - until the shared evidence base is consistent. Scope: multiple product areas share one coherent picture of the customer.</t>
+          <t>Depth: Independently frames ambiguous problems, selects fitting methods, and separates signal from noise. Evidenced by: Writes an insight document that changes the team's next quarter's plan, and a skeptical peer checking the chain from quote to claim finds it intact. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the org's insight infrastructure - repositories, tagging conventions, and synthesis reviews - so findings compound across teams instead of evaporating per project. Scope: product org.</t>
+          <t>Depth: Designs the team's discovery approach and untangles findings others find contradictory. Evidenced by: Notices two teams' research write-ups draw opposite conclusions about the same customer segment and runs the joint review that reconciles them into one shared picture. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Distills company-wide customer understanding into the few durable insights executives and boards reason from, and retires folklore that no longer survives the evidence. Scope: company portfolio.</t>
+          <t>Depth: Sets the org's research strategy and anticipates emerging customer needs before they surface. Evidenced by: Stands up the org's tagging conventions and insight repository so a finding from one team's research is discoverable and reusable by another team a year later. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what rigorous product discovery means and shapes the discipline's practice externally. Evidenced by: Distills a year of company-wide customer research into the handful of insights the executive team actually reasons from, and retires a piece of long-standing but unsupported folklore. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1020,37 +1046,42 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Cooper, *The Inmates Are Running the Asylum* (1999)</t>
+          <t>Mapping target segments and their end-to-end experiences to ground product decisions.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Uses the team's personas and segments correctly in specs and interview recruiting - names which persona a story serves, and flags work that serves no one in particular. Scope: one epic's user definitions.</t>
+          <t>Cooper, Reimann, Cronin &amp; Noessel, About Face: The Essentials of Interaction Design, 4th Edition (Wiley, 2014) — substituted for Cooper's The Inmates Are Running the Asylum (no bibliography entry) with Cooper, Reimann, Cronin &amp; Noessel's About Face, the same author's canonical goal-directed-design text that originated the persona method Inmates popularized; adoption is won segment by segment, per Moore's chasm model.</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps their area's personas and segments evidence-based - refreshes them from interview and usage data, splits a segment when behavior diverges, and retires personas that no longer match observed users. Scope: their product area's segmentation.</t>
+          <t>Depth: Documents personas and journey steps from supplied data under direction. Evidenced by: Names which persona a new user story serves when writing it, and flags a proposed feature in review as serving no defined segment. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Chooses the target segment for their product deliberately and defends it - names who the product is not for, sizes segments with data, and maps the end-to-end journey per segment so gaps become visible. Scope: their product; design and marketing build from their segment definitions.</t>
+          <t>Depth: Builds usable personas and maps journeys for a product area with normal review. Evidenced by: Refreshes their product area's personas from a quarter of new interview and usage data, splitting one persona into two once their behavior clearly diverges. Scope: a product area.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reconciles segment and persona models across teams so the portfolio addresses one coherent map of users rather than overlapping caricatures. Scope: multiple product areas.</t>
+          <t>Depth: Independently models complex multi-actor journeys and resolves conflicting user signals. Evidenced by: Names, in a strategy review, exactly who the product is not building for this year, and backs the target-segment choice with sizing data the team can defend. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns the org's customer model - the shared segmentation the org plans, staffs, and measures against - and audits products for segment drift. Scope: product org.</t>
+          <t>Depth: Defines modeling standards others adopt and reconciles personas across overlapping segments. Evidenced by: Reconciles two product areas' persona sets that had quietly drifted into describing the same underlying user two different ways, and gets both teams onto one shared map. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines how the company sees its market's customers - the segment map used in company strategy and board materials - and updates it ahead of market shifts. Scope: company portfolio.</t>
+          <t>Depth: Sets persona and journey strategy across the portfolio and predicts shifting behavior patterns. Evidenced by: Owns the org's customer segmentation model and flags a product whose recent roadmap has drifted from the segment it was originally built for. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Establishes industry-recognized methods for journey modeling and teaches them widely. Evidenced by: Updates the company's customer segment map ahead of a market shift that board materials and company strategy then get built around. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1077,37 +1108,42 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Perri, *Escaping the Build Trap* (2018)</t>
+          <t>Frames incoming requests and observations as customer problems tied to measurable outcomes — separating the problem from the proposed solution before work is committed.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes a one-page problem statement naming the user, the struggle, and the evidence - and separates the problem from the requested feature when a stakeholder hands them a solution. Scope: one epic.</t>
+          <t>Perri, Escaping the Build Trap: How Effective Product Management Creates Real Value (O'Reilly, 2018) — teams stuck shipping outputs need problems framed as customer/business outcomes; self-sourced capability (PM-16 minted 2026-07 from this ladder's own prior consolidation prose — see scope_note), so evidence is written fresh below.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Frames work as outcomes the team can move ("reduce time-to-first-value") rather than outputs to ship, and rewrites incoming feature requests into the underlying problem before triage. Scope: their product area's backlog.</t>
+          <t>Depth: Writes a one-page problem statement naming the user, the struggle, and the evidence, with review; separates problem from requested feature when prompted. Evidenced by: Writes a one-page problem statement naming the user, the struggle, and the evidence for their epic, and a reviewer catches where it still smuggles in a feature. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the outcome their product is accountable for and keeps the team pointed at it, publicly re-framing efforts that drift into output-counting. Scope: their product; the problem framing survives their absence in planning docs.</t>
+          <t>Depth: Frames work as outcomes the team can move rather than outputs to ship, and rewrites incoming feature requests into the underlying problem before triage. Evidenced by: Rewrites an incoming stakeholder feature request into the underlying problem before it reaches triage, framing the goal as a movable number rather than a shipped artifact. Scope: a product area.</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Arbitrates problem framing across teams - spots when two areas are solving the same problem differently or optimizing conflicting outcomes, and reconciles the framing. Scope: multiple product areas.</t>
+          <t>Depth: Sets the outcome a product is accountable for and keeps the team pointed at it, publicly re-framing efforts that drift into output-counting. Evidenced by: Names, in a planning review, that the team has drifted into counting shipped tickets instead of moving the outcome it owns, and resets the conversation to the number that matters. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines the outcome architecture of the product org - how team-level outcomes ladder to product-level results - and retires vanity outcomes that don't. Scope: product org.</t>
+          <t>Depth: Arbitrates problem framing across teams — spotting duplicated or conflicting framings — and re-cuts problem boundaries drawn along org lines instead of customer lines. Evidenced by: Notices two product areas have quietly defined the same customer problem two incompatible ways and gets both teams working from one reconciled framing. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Frames the company's hardest, most ambiguous product problems - the ones with no owner - into tractable outcome statements executives fund. Scope: company portfolio.</t>
+          <t>Depth: Defines an organization's outcome architecture — how team-level outcomes ladder to organizational results — and retires vanity outcomes. Evidenced by: Publishes how team-level outcomes ladder up to the product org's results, and retires a long-tracked metric that turned out to be a vanity number nobody could act on. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Frames an organization's hardest, ownerless problems into tractable outcome statements executives fund; their framing practice shapes the discipline externally. Evidenced by: Takes a company-level problem with no clear owner — churn nobody's roadmap addresses — and frames it into an outcome statement executives fund and a team is staffed against. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1134,37 +1170,42 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Christensen, Hall, Dillon &amp; Duncan, *Competing Against Luck* (2016)</t>
+          <t>Models what customers hire products to accomplish — the circumstance, the progress sought, and the competing alternatives (including workarounds and non-consumption) — to predict adoption and define product boundaries.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Restates a feature request as the job the customer is hiring it for, including the circumstance and the progress sought, with coaching on the functional/emotional/social split. Scope: individual requests on one feature.</t>
+          <t>Christensen, Hall, Dillon &amp; Duncan, Competing Against Luck: The Story of Innovation and Customer Choice (HarperBusiness, 2016) — customers hire products to make progress in a circumstance; self-sourced capability (PM-17 minted 2026-07 from this ladder's own prior consolidation prose — see scope_note), so evidence is written fresh below.</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Maps the main jobs in their area from interview evidence, identifying what customers currently hire (including non-consumption and workarounds) and where those hires fail. Scope: their product area.</t>
+          <t>Depth: Restates a feature request as the job the customer is hiring it for — circumstance and progress sought — with coaching. Evidenced by: Restates a stakeholder's feature request as the job the customer is hiring it for — the circumstance and the progress sought — after a lead points out the request was solution-shaped. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Anchors their product's definition and boundaries in its core job, using the job to rule scope in or out and to identify non-obvious competitors. Scope: their product; the job statement appears in the team's strategy doc, in their words.</t>
+          <t>Depth: Maps the main jobs in their area from interview evidence, identifying what customers currently hire and where those hires fail. Evidenced by: Maps the three or four jobs customers hire their product area for from a batch of interviews, and names where a current job is being served badly enough that customers work around it. Scope: a product area.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Aligns job maps across areas into one view of customer progress, exposing where the portfolio makes customers stitch products together to finish one job. Scope: multiple product areas.</t>
+          <t>Depth: Anchors a product's definition and boundaries in its core job, using the job to rule scope in or out and to identify non-obvious competitors. Evidenced by: Rules a proposed feature out of scope because it does not advance the product's core job, and names a competitor outside the product's category that serves the same job better. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Uses jobs analysis to shape org-level portfolio choices - which jobs the org serves end-to-end, which it exits - in documents the leadership team debates from. Scope: product org.</t>
+          <t>Depth: Aligns job maps across teams into one view of customer progress, exposing where customers must stitch products together to finish one job. Evidenced by: Aligns two teams' separate job maps into one view and shows where customers currently stitch both teams' products together to finish a single job neither owns end to end. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Frames company strategy in jobs terms that reveal disruption threats and adjacent-market entries before the market makes them obvious. Scope: company portfolio.</t>
+          <t>Depth: Uses jobs analysis to shape organization-level portfolio choices — which jobs are served end-to-end, which are exited. Evidenced by: Uses a jobs-based view of the portfolio to recommend exiting a product line that serves a job the company can no longer serve better than the alternatives customers already use. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Frames markets and strategy in jobs terms that reveal disruption threats early; their jobs analyses influence practice beyond their organization. Evidenced by: Frames an emerging market shift in jobs terms that flags a disruption threat before competitors name it, and the analysis gets cited by other companies watching the same market. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1191,37 +1232,42 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Bland &amp; Osterwalder, *Testing Business Ideas* (2019); Cagan, *Inspired* (2nd ed., 2018)</t>
+          <t>Names and ranks the assumptions behind a product bet — desirability, viability, feasibility, usability — and designs the cheapest decisive pre-build tests (prototypes, fake doors, concierge runs) to validate or kill them.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Lists the assumptions behind their epic and sorts them by importance and evidence, using the four-risks lens with coaching. Scope: one epic's risk map.</t>
+          <t>Bland &amp; Osterwalder, Testing Business Ideas: A Field Guide for Rapid Experimentation (Wiley, 2019) — desirability, viability, feasibility, and usability risks must be named and ranked before building, paired with Cagan's four discovery risks; self-sourced capability (PM-18 minted 2026-07 from this ladder's own prior consolidation prose — see scope_note), so evidence is written fresh below.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Identifies the riskiest assumption before any build starts and says so in planning, choosing what to test first rather than testing what is easiest. Scope: their area's bets.</t>
+          <t>Depth: Lists the assumptions behind a proposed feature, sorts them by risk with coaching, and runs a prescribed simple test, logging what was learned. Evidenced by: Lists the desirability, viability, feasibility, and usability assumptions behind a proposed feature with a lead's coaching, and runs the one prescribed prototype test the lead assigned. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Surfaces the assumptions others treat as facts - in their own bets and in reviews of others' - and kills initiatives whose load-bearing assumptions fail. Scope: a product's risk discipline; their pre-mortems are copied.</t>
+          <t>Depth: Identifies the riskiest assumption before build and matches the test type to it — prototype, painted door, concierge — with pass/fail defined in advance. Evidenced by: Names the riskiest assumption in a proposed bet before any build starts, picks a painted-door test to match it, and writes down the pass/fail bar before launching it. Scope: a product area.</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Standardizes how multiple teams express and rank risk so bets are comparable across areas, and challenges cross-team initiatives carrying untested compound assumptions. Scope: multiple product areas.</t>
+          <t>Depth: Surfaces assumptions others treat as facts, designs test sequences that retire the most risk per unit effort, and kills initiatives whose load-bearing assumptions fail. Evidenced by: Kills an initiative in flight after a pre-mortem surfaces a load-bearing assumption the team had been quietly treating as a fact, naming the evidence and the trade-off in the write-up. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds risk review into the org's investment process - big funding asks arrive with assumption maps or go back - and calibrates the org's risk appetite explicitly. Scope: product org.</t>
+          <t>Depth: Standardizes how multiple teams express and rank risk, and rejects validation theater — tests that can only confirm, never falsify — before major commitments. Evidenced by: Standardizes how three teams express and compare risk on their bets and rejects a test design that could only ever confirm the team's existing plan. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Stress-tests portfolio bets' foundational assumptions in executive forums, naming the belief that would have to be true and what evidence exists for it. Scope: company portfolio.</t>
+          <t>Depth: Builds discovery-testing capability into an organization's investment process — funding follows tested assumptions, and the cost of a first test drops to hours. Evidenced by: Gets the org's investment process to require a tested-assumption map before funding a major bet, dropping the cost of a first test from weeks to hours. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Structures bets too big to A/B as staged, falsifiable commitments; their validation doctrine is cited and adopted beyond their organization. Evidenced by: Structures a bet too large to A/B — a new pricing model — as a sequence of staged, falsifiable commitments, and other companies cite the approach when facing similar bets. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1248,37 +1294,42 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Ries, *The Lean Startup* (2011); Torres, *Continuous Discovery Habits* (2021)</t>
+          <t>Names and ranks the assumptions behind a product bet — desirability, viability, feasibility, usability — and designs the cheapest decisive pre-build tests (prototypes, fake doors, concierge runs) to validate or kill them.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds simple tests - fake-door links, clickable prototypes, concierge runs - from a design someone else specified, and logs what was learned. Scope: one assumption at a time.</t>
+          <t>Ries, The Lean Startup: How Today's Entrepreneurs Use Continuous Innovation to Create Radically Successful Businesses (Crown Business, 2011) — the smallest test that produces validated learning beats the most polished untested build, paired with Torres's continuous-testing habit; self-sourced capability (PM-18 minted 2026-07 from this ladder's own prior consolidation prose — see scope_note), so evidence is written fresh below.</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Chooses the test type that matches the assumption - prototype for usability, painted door for demand, Wizard of Oz for feasibility - and defines pass/fail before launching it. Scope: their area's assumption tests.</t>
+          <t>Depth: Lists the assumptions behind a proposed feature, sorts them by risk with coaching, and runs a prescribed simple test, logging what was learned. Evidenced by: Builds a fake-door test from a design a senior PM already specified, launches it exactly as instructed, and logs what the click-through data showed. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs test sequences that retire the most risk per week of effort, and rejects tests whose result couldn't change the decision. Scope: a product; their test designs are the examples in onboarding.</t>
+          <t>Depth: Identifies the riskiest assumption before build and matches the test type to it — prototype, painted door, concierge — with pass/fail defined in advance. Evidenced by: Picks a painted-door test to check demand for a proposed feature, defines the click-through rate that counts as a pass before launching it, and reports the result honestly when it fails. Scope: a product area.</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Unblocks teams whose experiments keep coming back inconclusive, redesigning the test rather than rerunning it bigger. Scope: multiple product areas.</t>
+          <t>Depth: Surfaces assumptions others treat as facts, designs test sequences that retire the most risk per unit effort, and kills initiatives whose load-bearing assumptions fail. Evidenced by: Designs a sequence of three cheap tests that retires the two riskiest assumptions behind a bet in a week, and cancels a fourth test whose result couldn't have changed the team's decision either way. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the org's testing toolkit - reusable painted-door infrastructure, prototype panels, templates - dropping the cost of a first test to hours. Scope: product org.</t>
+          <t>Depth: Standardizes how multiple teams express and rank risk, and rejects validation theater — tests that can only confirm, never falsify — before major commitments. Evidenced by: Redesigns another team's third inconclusive prototype test — the problem was the test, not the users — instead of letting them rerun the same test at larger scale. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs validation for bets too big to A/B - new markets, pricing models, platforms - using staged commitments and falsifiable milestones. Scope: company portfolio.</t>
+          <t>Depth: Builds discovery-testing capability into an organization's investment process — funding follows tested assumptions, and the cost of a first test drops to hours. Evidenced by: Builds a shared prototype-testing panel and painted-door toolkit that drops the org's cost of a first test from a two-week build to an afternoon. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Structures bets too big to A/B as staged, falsifiable commitments; their validation doctrine is cited and adopted beyond their organization. Evidenced by: Designs a staged, falsifiable validation plan for a bet on an entirely new pricing model too large to A/B, with milestones the company can kill the bet against. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1305,37 +1356,42 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Olsen, *The Lean Product Playbook* (2015)</t>
+          <t>Names and ranks the assumptions behind a product bet — desirability, viability, feasibility, usability — and designs the cheapest decisive pre-build tests (prototypes, fake doors, concierge runs) to validate or kill them.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs moderated tests of an existing prototype from a task script, noting where users struggle without explaining the design to them. Scope: usability of one feature.</t>
+          <t>Bland &amp; Osterwalder, Testing Business Ideas: A Field Guide for Rapid Experimentation (Wiley, 2019) — substituted for Olsen's The Lean Product Playbook (no bibliography entry) with Bland &amp; Osterwalder's experiment library, which explicitly includes prototype and solution tests; self-sourced capability (PM-18 minted 2026-07 from this ladder's own prior consolidation prose — see scope_note), so evidence is fresh below.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Pairs with design to build the right-fidelity prototype for the question at hand and iterates it between test rounds, reporting what changed and why. Scope: solution tests across their product area.</t>
+          <t>Depth: Lists the assumptions behind a proposed feature, sorts them by risk with coaching, and runs a prescribed simple test, logging what was learned. Evidenced by: Runs a moderated usability test of an existing clickable prototype from a task script a designer wrote, noting where the participant stalls without explaining the design to them. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Chooses the testing method by risk - prototype, Wizard-of-Oz, live-data test - and calls when the evidence is sufficient to commit to build. Scope: their product; design partners treat them as a peer in test planning.</t>
+          <t>Depth: Identifies the riskiest assumption before build and matches the test type to it — prototype, painted door, concierge — with pass/fail defined in advance. Evidenced by: Pairs with design to build a low-fidelity prototype that matches the question at hand, tests it with five users, and reports what changed between rounds and why. Scope: a product area.</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reviews other teams' solution tests before major commitments and catches tests that can only confirm, never falsify. Scope: multiple product areas.</t>
+          <t>Depth: Surfaces assumptions others treat as facts, designs test sequences that retire the most risk per unit effort, and kills initiatives whose load-bearing assumptions fail. Evidenced by: Chooses live-data testing over a prototype for a bet where the real signal only shows up under real usage, and the team commits to build once the evidence is sufficient by a bar set in advance. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the org's prototyping-and-testing muscle - tooling, research-ops support, fidelity norms - so testing before building is the cheap default everywhere. Scope: product org.</t>
+          <t>Depth: Standardizes how multiple teams express and rank risk, and rejects validation theater — tests that can only confirm, never falsify — before major commitments. Evidenced by: Reviews another team's solution test ahead of a major commitment and catches that the test, as designed, could only ever confirm the team already wanted to build it. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Represents test-before-build as company doctrine, defending the practice when executive pressure pushes for committed roadmaps without evidence. Scope: company portfolio.</t>
+          <t>Depth: Builds discovery-testing capability into an organization's investment process — funding follows tested assumptions, and the cost of a first test drops to hours. Evidenced by: Builds the org's shared prototyping panel and fidelity norms so every team's default is to test a solution cheaply before committing engineering time to it. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Structures bets too big to A/B as staged, falsifiable commitments; their validation doctrine is cited and adopted beyond their organization. Evidenced by: Represents test-before-build as company doctrine in front of executives pushing for a committed roadmap without evidence, and the practice holds. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1362,37 +1418,42 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Rumelt, *Good Strategy Bad Strategy* (2011)</t>
+          <t>Defining target markets, value propositions, and differentiation that guide what to build and why.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Explains their team's strategy in their own words and connects their epic's work to it when asked. Scope: consumes strategy for one epic.</t>
+          <t>Rumelt, Good Strategy Bad Strategy: The Difference and Why It Matters (Crown Business, 2011) — real strategy is diagnosis, guiding policy, and coherent action; most "strategies" are goals, and the craft is the diagnosis that names the real obstacle before choosing what to do about it.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Derives their area's priorities from the product strategy explicitly, writing them down as choices - what they are doing and what they are explicitly not - and flags work that doesn't serve it. Scope: a product area.</t>
+          <t>Depth: Drafts positioning statements from a given strategy under direction. Evidenced by: Drafts the positioning statement for their epic from the strategy their lead already set, and revises it twice on review before it holds up. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes the strategy for their product - a diagnosis, a guiding policy, and the coherent bets - and defends the kill-list it implies in front of the stakeholders who asked. Scope: owns strategy for a product; the team quotes the strategy when declining work.</t>
+          <t>Depth: Articulates strategy and positioning for one product with normal review. Evidenced by: Writes down their product area's priorities as explicit choices — what they are doing and what they are deliberately not — and flags a request that doesn't serve the stated strategy. Scope: a product area.</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes strategies other PMs adopt as the frame for their own areas, and reviews area strategies for incoherence between diagnosis and bets. Scope: multiple product areas.</t>
+          <t>Depth: Independently sets coherent strategy amid ambiguity and defends hard trade-offs. Evidenced by: Writes the diagnosis, guiding policy, and coherent bets for their product's strategy, and defends the resulting kill-list to the stakeholders who proposed the killed work. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes the product org's strategy - where to concentrate, what to starve - in documents leadership funds against. Scope: product organization.</t>
+          <t>Depth: Defines the strategy framework teams adopt and resolves conflicting strategic bets. Evidenced by: Writes a strategy framework that two other product teams adopt as the frame for their own areas, and reviews a peer's area strategy for a diagnosis that doesn't match its stated bets. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Co-authors company strategy from the product side, and the portfolio's shape reflects arguments they made. Scope: company portfolio.</t>
+          <t>Depth: Owns portfolio-level strategy and anticipates where the market is heading. Evidenced by: Shapes where the product org concentrates investment and where it deliberately starves a line, in a document leadership funds against. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what good product strategy means for the discipline and influences practice externally. Evidenced by: Co-authors the company's strategy from the product side, and the shape of the portfolio a year later reflects arguments made in that document. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1419,37 +1480,42 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Dunford, *Obviously Awesome* (2019); Moore, *Crossing the Chasm* (3rd ed., 2014)</t>
+          <t>Defining target markets, value propositions, and differentiation that guide what to build and why.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Depth: States who the product is for, what it replaces, and why it wins in two sentences consistent with the team's positioning canvas. Scope: describes their feature's value accurately.</t>
+          <t>Dunford, Obviously Awesome: How to Nail Product Positioning (Ambient Press, 2019) — deliberate positioning against the right competitive alternatives determines whether strengths read as value, paired with Moore's chasm-crossing model of adoption won segment by segment.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Maintains the positioning for their area - target segment, competitive alternatives, differentiated value - and flags when a proposed feature blurs it. Scope: a product area's positioning artifacts.</t>
+          <t>Depth: Drafts positioning statements from a given strategy under direction. Evidenced by: States who a new feature is for, what it replaces, and why it wins in two sentences that match the team's existing positioning canvas. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Repositions a product deliberately when the market shifts, running the analysis of alternatives and trade-offs in writing; marketing builds messaging from their positioning work. Scope: a product; sales and marketing treat their positioning doc as source of truth.</t>
+          <t>Depth: Articulates strategy and positioning for one product with normal review. Evidenced by: Flags in review that a proposed feature would blur their area's positioning against a named competitive alternative, and gets the scope adjusted before it ships. Scope: a product area.</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps positioning coherent across a product family, resolving where products in the portfolio overlap, undercut, or contradict each other in-market. Scope: multiple product areas.</t>
+          <t>Depth: Independently sets coherent strategy amid ambiguity and defends hard trade-offs. Evidenced by: Repositions a product after a competitor's launch shifts the market, running the alternatives analysis in writing, and marketing builds the next campaign from that document. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org's differentiation strategy - which capabilities the org will be known for and which it deliberately concedes - and holds roadmaps to it. Scope: product org.</t>
+          <t>Depth: Defines the strategy framework teams adopt and resolves conflicting strategic bets. Evidenced by: Resolves a case where two products in the same family were quietly undercutting each other's positioning in sales conversations, and issues one coherent family positioning doc. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Positions the company itself - category creation or category redefinition arguments that analysts and competitors respond to. Scope: company portfolio and market narrative.</t>
+          <t>Depth: Owns portfolio-level strategy and anticipates where the market is heading. Evidenced by: Sets which capabilities the org will be known for this year and which it will deliberately not compete on, and holds two roadmaps to that line when they drift. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what good product strategy means for the discipline and influences practice externally. Evidenced by: Makes the category-redefinition argument that gets picked up by industry analysts covering the company's market. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1476,37 +1542,42 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Cagan, *Inspired* (2nd ed., 2018)</t>
+          <t>Articulating product vision and outcome-based objectives that align teams over time.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Retells the product vision accurately and uses it to answer "why are we building this" for their epic. Scope: one epic.</t>
+          <t>Cagan, INSPIRED: How to Create Tech Products Customers Love, 2nd Edition (Wiley, 2018) — a compelling product vision recruits, aligns, and outlasts individual roadmaps; teams need a destination that survives quarterly churn.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Connects their area's roadmap to the vision in planning docs, noticing when proposed work leads away from it, and aligns their team and stakeholders behind it. Scope: a product area.</t>
+          <t>Depth: Translates a stated vision into concrete goals under direction. Evidenced by: Explains to a new teammate why their epic matters by retelling the product vision accurately, without needing the lead to translate it. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes a vision narrative (visiontype, storyboard, or press-release-style doc) that teams reference months later when making local decisions. Scope: a product's vision; engineers and designers cite it unprompted.</t>
+          <t>Depth: Sets clear, measurable goals for a product area with normal review. Evidenced by: Points out in a planning review that a proposed feature leads the roadmap away from the stated vision, and gets the team realigned before committing the sprint. Scope: a product area.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Crafts vision artifacts that align several products toward one future, resolving contradictions between area visions before they become shipped contradictions. Scope: multiple product areas.</t>
+          <t>Depth: Independently crafts a compelling vision and cascades aligned goals through ambiguity. Evidenced by: Writes a press-release-style vision doc that an engineer cites unprompted three months later to justify a local design decision. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns the product org's north-star narrative and refreshes it when the diagnosis changes, visibly retiring the old one. Scope: product organization.</t>
+          <t>Depth: Defines goal-setting frameworks others adopt and aligns competing visions. Evidenced by: Writes a vision artifact that resolves a contradiction between two product areas' separate visions before either team ships something the other would have to walk back. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Articulates the company's product future in narratives used for recruiting, fundraising, and board alignment. Scope: company portfolio.</t>
+          <t>Depth: Sets enduring vision across the portfolio and anticipates long-horizon shifts. Evidenced by: Owns the product org's north-star narrative and visibly retires it in favor of a new one once the underlying diagnosis has changed. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes how the discipline frames product vision and is externally credible on it. Evidenced by: Writes the product future narrative used in the company's fundraising deck and cited in board discussions of where the company is headed. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1533,37 +1604,42 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Perri, *Escaping the Build Trap* (2018); Lombardo, McCarthy, Ryan &amp; Connors, *Product Roadmaps Relaunched* (2017)</t>
+          <t>Sequencing initiatives across products and horizons against goals, capacity, and dependencies.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps their epic's roadmap entry current - status, confidence, what was learned - and explains to stakeholders why items are time-horizoned rather than dated. Scope: one epic's slice of the roadmap.</t>
+          <t>Perri, Escaping the Build Trap: How Effective Product Management Creates Real Value (O'Reilly, 2018) — roadmaps as strategic communication of outcomes and confidence, not feature release calendars, paired with Lombardo et al.'s theme-based, now/next/later roadmap format that operationalizes the same idea.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds their area's roadmap around outcomes with now/next/later horizons and explicit confidence levels, resisting stakeholder pressure to convert it into a promise list. Scope: their product area.</t>
+          <t>Depth: Maintains roadmap items and updates status under guidance. Evidenced by: Keeps their epic's roadmap entry current — status, confidence, what was learned — and explains to a stakeholder why it shows a quarter, not a date. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs the roadmap as a strategic negotiation - trades scope against outcomes with leadership, and shows in review how roadmap changes trace to discovery evidence. Scope: their product; sales and CS plan against their roadmap without being burned.</t>
+          <t>Depth: Builds and sequences a credible roadmap for one product with normal review. Evidenced by: Builds their product area's now/next/later roadmap around outcomes and holds the line when a stakeholder pushes to convert 'later' into a committed date. Scope: a product area.</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Aligns roadmaps across areas into a coherent sequence, surfacing cross-team dependencies and outcome conflicts before they collide in delivery. Scope: multiple product areas.</t>
+          <t>Depth: Independently balances competing priorities and replans confidently under shifting constraints. Evidenced by: Trades scope for outcome with a VP in a roadmap review and shows, in the same meeting, exactly which discovery evidence justifies the change from last quarter's plan. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns the org's roadmap process - cadence, format, confidence language - and defends outcome framing when executives ask for date certainty the evidence can't support. Scope: product org.</t>
+          <t>Depth: Designs the planning approach others use and resolves cross-team portfolio conflicts. Evidenced by: Surfaces a dependency between two areas' roadmaps that would have collided mid-quarter and re-sequences both before either team commits the conflicting work. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Presents the portfolio roadmap to boards and top customers as a strategy narrative, and sets the company norm for what roadmaps do and don't commit. Scope: company portfolio.</t>
+          <t>Depth: Sets portfolio planning strategy and foresees where investment should shift next. Evidenced by: Owns the cadence and confidence-language format every product team's roadmap uses, and defends the now/next/later structure when an executive asks for firm dates the evidence can't support. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines portfolio-planning best practice for the field and is recognized for it. Evidenced by: Presents the company's portfolio roadmap to the board as a strategy narrative, and sets the company-wide norm for what a roadmap does and doesn't promise. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1590,37 +1666,42 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Doerr, *Measure What Matters* (2018)</t>
+          <t>Articulating product vision and outcome-based objectives that align teams over time.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes measurable key results for their epic that describe user/business change rather than shipping ("activation +5pts" not "launch onboarding"), with review. Scope: one epic's goals.</t>
+          <t>Doerr, Measure What Matters (Portfolio/Penguin, 2018) — objectives with measurable key results align effort and expose sandbagging; goals are the interface between strategy and weekly work.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets their area's quarterly OKRs and grades them honestly at quarter end, separating "we shipped it" from "it worked" in the retro. Scope: their product area.</t>
+          <t>Depth: Translates a stated vision into concrete goals under direction. Evidenced by: Writes a measurable key result for their epic that names a user or business change rather than a shipped artifact, with a lead's review catching the first draft's vanity metric. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Negotiates their product's goals up and down the ladder - pushes back on cascaded targets the evidence can't support, and re-scopes mid-quarter when a key result is learned to be wrong. Scope: their product; their goal reviews are where the team's real trade-offs get made.</t>
+          <t>Depth: Sets clear, measurable goals for a product area with normal review. Evidenced by: Sets their product area's quarterly OKRs, and at quarter end grades honestly that a key result was hit but the underlying goal wasn't actually moved. Scope: a product area.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reviews goal quality across teams, catching output-dressed-as-outcome and metrics teams can't actually influence, and coaches the rewrite. Scope: multiple product areas.</t>
+          <t>Depth: Independently crafts a compelling vision and cascades aligned goals through ambiguity. Evidenced by: Pushes back on a cascaded target the team's own evidence doesn't support, and re-scopes a key result mid-quarter once new data shows the original one was set wrong. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs the org's goal architecture - how product OKRs ladder to company results without becoming a cascade of fiction - and runs the calibration where conflicts get resolved. Scope: product org.</t>
+          <t>Depth: Defines goal-setting frameworks others adopt and aligns competing visions. Evidenced by: Reviews a peer's team's OKRs, catches a key result that's really an output count in disguise, and coaches the rewrite into something the team can actually be judged against. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes company-level objectives and the discipline around them, holding the line on measurable outcomes at the executive table. Scope: company portfolio.</t>
+          <t>Depth: Sets enduring vision across the portfolio and anticipates long-horizon shifts. Evidenced by: Designs how product-team OKRs ladder to company-level results without becoming a chain of restated numbers, and runs the calibration session where two teams' conflicting goals get resolved. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes how the discipline frames product vision and is externally credible on it. Evidenced by: Holds the line on measurable, outcome-based objectives at the executive table when a leader proposes a vague, unmeasurable company goal for the year. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1647,37 +1728,42 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Croll &amp; Yoskovitz, *Lean Analytics* (2013)</t>
+          <t>Defining success metrics and interpreting product data to evaluate impact and guide iteration.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines success and guardrail metrics for their feature before build starts and states how each will be instrumented, distinguishing a vanity count from an actionable rate with guidance. Scope: one feature's metric set.</t>
+          <t>Croll &amp; Yoskovitz, Lean Analytics: Use Data to Build a Better Startup Faster (O'Reilly, 2013) — the One Metric That Matters and the vanity-metric critique; a product optimizes whatever its metrics reward, so metric design is behavior design.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns their area's metrics tree - how feature metrics roll to the area's north-star input - and retires metrics that move without meaning anything. Scope: their product area's dashboard, which they built or specified.</t>
+          <t>Depth: Pulls and reports defined product metrics under direction. Evidenced by: Pulls and reports the metrics their lead already defined for a launched feature, distinguishing a vanity count from an actionable rate with guidance when asked. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs the metric their product is judged by and defends its trade-offs (gameability, lag, proxy distance from value) when leadership wants a friendlier number. Scope: their product; other functions report against metrics this person defined.</t>
+          <t>Depth: Builds and interprets metric dashboards for a product with normal review. Evidenced by: Builds and owns the dashboard for their product area's metrics tree, retiring a metric that had been moving without anyone able to say why it mattered. Scope: a product area.</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reconciles metric definitions across teams so "activation" means one thing everywhere, and reviews new metrics for perverse incentives before they ship. Scope: multiple product areas.</t>
+          <t>Depth: Independently designs metric frameworks and draws sound conclusions from messy data. Evidenced by: Designs the single metric their product is judged by and defends, to a leadership team wanting a friendlier number, why the current one is the honest one despite the bad quarter it's showing. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org's measurement standards - north-star framework, guardrail policy, instrumentation quality bar - and audits whether dashboards reflect reality. Scope: product org.</t>
+          <t>Depth: Defines the measurement model teams adopt and diagnoses misleading metrics others trust. Evidenced by: Reconciles three teams' different definitions of 'activation' into one shared definition, and catches a proposed new metric that would reward a perverse shortcut before it ships. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines how the company measures product success at portfolio level, connecting product metrics to financial outcomes in models the CFO's team uses. Scope: company portfolio.</t>
+          <t>Depth: Sets product-analytics strategy across the org and anticipates which signals will matter. Evidenced by: Sets the org's north-star metric framework and guardrail policy, and audits a team's dashboard that turns out not to reflect what's actually happening with users. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines rigorous product measurement for the discipline and is cited externally on it. Evidenced by: Defines how the company connects product metrics to financial outcomes in a model the finance team uses directly in board reporting. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1704,37 +1790,42 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>McClure, "Startup Metrics for Pirates" (AARRR, 2007); Croll &amp; Yoskovitz, *Lean Analytics* (2013)</t>
+          <t>Defining success metrics and interpreting product data to evaluate impact and guide iteration.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Pulls their own funnel and retention numbers using the analytics stack, and describes what the data shows without inferring cause from correlation. Scope: their feature's usage data.</t>
+          <t>Croll &amp; Yoskovitz, Lean Analytics: Use Data to Build a Better Startup Faster (O'Reilly, 2013) — substituted (McClure's 'Startup Metrics for Pirates' has no bibliography entry) with the anchor already carried above: Croll &amp; Yoskovitz's stage-based funnel and cohort model incorporates AARRR directly and is already in the bibliography.</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs cohort and segmentation analyses that locate where their area leaks value, and pairs the quantitative "where" with qualitative "why" before proposing fixes. Scope: a product area's behavioral picture.</t>
+          <t>Depth: Pulls and reports defined product metrics under direction. Evidenced by: Pulls their feature's funnel numbers from the analytics stack and reports the drop-off honestly without guessing at a cause the data doesn't show. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Catches analytical traps in their own and others' analyses - survivorship, seasonality, mix shifts, Simpson's paradox - and their read of ambiguous data settles debates. Scope: a product; teams bring them analyses for sanity-checking.</t>
+          <t>Depth: Builds and interprets metric dashboards for a product with normal review. Evidenced by: Runs a cohort analysis that locates exactly which step of their area's funnel is leaking value, then pairs it with a handful of interviews to explain why before proposing a fix. Scope: a product area.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Traces customer journeys across product boundaries, quantifying cross-product friction no single team's dashboard shows. Scope: multiple product areas.</t>
+          <t>Depth: Independently designs metric frameworks and draws sound conclusions from messy data. Evidenced by: Catches that a colleague's promising-looking retention chart is a seasonality artifact, not a real improvement, before it gets presented as a win. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org's analytical standards and self-serve tooling priorities so teams answer their own questions correctly without a data-science queue. Scope: product org.</t>
+          <t>Depth: Defines the measurement model teams adopt and diagnoses misleading metrics others trust. Evidenced by: Traces a customer journey that crosses two products' boundaries and quantifies friction — a re-login, a re-entered form — that neither team's own dashboard was built to show. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reads portfolio-level behavioral shifts early - usage patterns that presage churn, expansion, or disruption - and gets the company to act on them. Scope: company portfolio.</t>
+          <t>Depth: Sets product-analytics strategy across the org and anticipates which signals will matter. Evidenced by: Builds the org's self-serve analytics tooling so teams can answer their own funnel questions correctly without waiting on a data-science queue. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines rigorous product measurement for the discipline and is cited externally on it. Evidenced by: Spots an early portfolio-level usage shift that presages churn in a major segment months before it shows up in revenue, and gets the company to act on it. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1761,37 +1852,42 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Kohavi, Tang &amp; Xu, *Trustworthy Online Controlled Experiments* (2020)</t>
+          <t>Designing and reading controlled experiments to validate hypotheses and de-risk decisions.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes a test plan with hypothesis, primary metric, and minimum sample worked out with an analyst, and waits for the pre-agreed end date before reading results. Scope: one feature's experiments.</t>
+          <t>Kohavi, Tang &amp; Xu, Trustworthy Online Controlled Experiments: A Practical Guide to A/B Testing (Cambridge University Press, 2020) — controlled experiments as the gold standard for causal claims, and the catalog of ways they silently lie (SRM, peeking, novelty effects).</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs and ships their own A/B tests correctly - power calculation, guardrail metrics, no peeking, no post-hoc metric shopping - and writes up null results as findings. Scope: their area's experiment pipeline.</t>
+          <t>Depth: Runs predefined experiments and records results under supervision. Evidenced by: Runs an A/B test exactly as an analyst designed it, records the results without touching the analysis method, and waits for the pre-agreed end date. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Catches invalid experiments before decisions get made on them - SRM, novelty effects, interaction between concurrent tests - and knows when an A/B test is the wrong instrument entirely. Scope: a product's experimentation quality; they are the reviewer of record for others' test designs.</t>
+          <t>Depth: Designs and analyzes a standard A/B test with normal review. Evidenced by: Designs and ships an A/B test for their own feature — power calculation, guardrail metrics, no peeking — and writes up a null result honestly instead of quietly shelving it. Scope: a product area.</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Audits experiment practice across teams, catching cherry-picked segments and re-run-until-significant patterns, and standardizes the readout format others adopt. Scope: multiple product areas.</t>
+          <t>Depth: Independently designs valid experiments and interprets ambiguous or conflicting results. Evidenced by: Catches a sample-ratio mismatch in a colleague's experiment before its result gets used to justify a launch, and is the person their own product's other PMs ask to sanity-check a test design before it ships. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the org's experimentation culture and platform requirements - institutional memory of past results, meta-analysis of what interventions work - so learning compounds. Scope: product org.</t>
+          <t>Depth: Defines experimentation standards others adopt and rescues flawed test designs. Evidenced by: Audits experiment practice across three teams, catches a pattern of rerunning tests until they hit significance, and gets one shared readout format adopted everywhere. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets company policy on evidence standards for product decisions, including where experimentation is mandatory and where judgment rightly overrides it. Scope: company portfolio.</t>
+          <t>Depth: Sets the org's experimentation strategy and anticipates where testing should expand. Evidenced by: Builds the org's experimentation platform requirements and a repository of past results so a new test doesn't reinvent an intervention that's already been tried and failed. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines experimentation rigor for the discipline and influences external practice. Evidenced by: Sets company policy on where A/B testing is mandatory before a launch and where judgment rightly overrides it, and the policy holds under executive pressure to skip it. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1818,37 +1914,42 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Duke, *Thinking in Bets* (2018)</t>
+          <t>Makes sound calls with incomplete information.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes down the options considered and the reasoning before a decision, and distinguishes a bad outcome from a bad decision in retros, with prompting. Scope: decisions within one epic.</t>
+          <t>Kahneman, Thinking, Fast and Slow (Farrar, Straus and Giroux, 2011) — substituted for Duke's Thinking in Bets (no bibliography entry) with Kahneman's Thinking, Fast and Slow, the other named source in the original two-author anchor line — the named biases that predictably distort product bets made under time pressure and incomplete information.</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Depth: States confidence levels and reversibility when deciding - moves fast on two-way doors, slows down on one-way doors - and keeps a decision log the team consults. Scope: their product area's calls.</t>
+          <t>Depth: Makes well-defined decisions; asks good questions when blocked. Evidenced by: Writes down the options considered and the reasoning before a decision on their epic, and separates a bad outcome from a bad decision in the retro when a lead prompts them to. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs decision-making the team trusts under pressure: names the disconfirming evidence, invites the strongest counter-argument, and changes course publicly when wrong. Scope: their product; escalations come to them because their reasoning is legible, not because of their title.</t>
+          <t>Depth: Decides independently within their components; evaluates alternatives honestly. Evidenced by: States their confidence level and whether a call is reversible before deciding, moving fast on the two-way doors and slowing down on the one-way ones, and keeps a decision log the team consults. Scope: a product area.</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reviews other PMs' consequential decisions pre-commitment, surfacing sunk-cost and confirmation patterns, and their decision-record format spreads across teams. Scope: multiple product areas.</t>
+          <t>Depth: Makes architectural choices for a domain that hold up over months. Evidenced by: Names the strongest disconfirming evidence against their own plan before a stakeholder can raise it, and changes course publicly once new data proves the original call wrong. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs the org's decision mechanisms - who decides what, at what evidence bar, with what escalation path - and runs pre-mortems on the biggest bets. Scope: product org.</t>
+          <t>Depth: Foresees second-order consequences; sets decision frameworks for teams. Evidenced by: Reviews another PM's high-stakes decision before it's committed, catches a sunk-cost pattern in the reasoning, and the decision-record format spreads to two other teams. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Is the judgment of last resort on company-level product calls, brought into ambiguous, high-stakes decisions precisely because their reasoning record is public and audited. Scope: company portfolio.</t>
+          <t>Depth: Sets decision-making frameworks for the org. Evidenced by: Designs the org's decision mechanism — who decides what, at what evidence bar, with what escalation path — and runs a pre-mortem on the year's biggest bet. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Visionary judgment; sees structural causes others miss. Evidenced by: Gets pulled into a company-level decision precisely because their reasoning record is public and audited, and their judgment settles a call nobody else could resolve. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1875,37 +1976,42 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Reinertsen, *The Principles of Product Development Flow* (2009)</t>
+          <t>Weighs cost, value, risk and timing.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Orders their epic's backlog with stated reasoning - value, urgency, dependency - and updates the order when facts change rather than defending it. Scope: one epic's backlog.</t>
+          <t>Reinertsen, The Principles of Product Development Flow: Second Generation Lean Product Development (Celeritas, 2009) — cost of delay divided by duration (WSJF) is the economically correct sequencing logic; intuition systematically misprices queues.</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Prioritizes across their whole area using an explicit method (cost of delay, RICE, or similar) and shows the math when stakeholders challenge the order. Scope: a product area's backlog.</t>
+          <t>Depth: Works highest-priority-first when told the priorities. Evidenced by: Orders their epic's backlog with stated reasoning — value, urgency, dependency — and re-orders it without protest when a lead points out a fact has changed. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Prioritizes across incommensurables - debt vs. features vs. compliance vs. bets - with written trade-off reasoning that stakeholders accept even when they lose. Scope: a product; their prioritization write-ups are the template others use.</t>
+          <t>Depth: Makes sound priority calls within scope; time-boxes uncertain work. Evidenced by: Prioritizes their product area's backlog using an explicit cost-of-delay estimate and shows the math when a stakeholder challenges the order. Scope: a product area.</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sequences investment across teams, moving scope between teams when the portfolio-level ordering demands it, with the displaced team's agreement on record. Scope: multiple product areas.</t>
+          <t>Depth: Balances cost/value/risk across a domain; resists hype; decisions hold up over months. Evidenced by: Sequences a quarter's work across debt, features, and a compliance deadline with written trade-off reasoning stakeholders accept even when their request loses. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes the org's resource allocation logic - the explicit framework by which the org funds run/grow/transform - and defends it through planning cycles. Scope: product org.</t>
+          <t>Depth: Expert at portfolio-level trade-offs; surfaces hidden assumptions; trusted tiebreaker. Evidenced by: Moves a chunk of scope from one team to another when the portfolio-level cost-of-delay math demands it, with the displaced team's agreement documented. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Influences portfolio-level capital allocation, making the economic case for which products get funded, harvested, or killed. Scope: company portfolio.</t>
+          <t>Depth: Sets decision frameworks for the org. Evidenced by: Builds the explicit framework the org uses to split investment across run, grow, and transform work, and defends it through a planning cycle that tries to override it. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Influences company strategic direction through judgment. Evidenced by: Makes the economic case that gets a product line harvested rather than continuing to be funded, using cost-of-delay reasoning the leadership team accepts. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1932,37 +2038,42 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Cagan, *Inspired* (2nd ed., 2018)</t>
+          <t>Slices work so value and learning arrive early.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Proposes which parts of their feature can ship later without breaking the core job, and writes the cut list with what's lost by each cut, for their lead to decide. Scope: one feature.</t>
+          <t>Cagan, INSPIRED: How to Create Tech Products Customers Love, 2nd Edition (Wiley, 2018) — deliver the smallest thing that achieves the outcome; the ability to cut scope without cutting the outcome is what separates shipping-on-time from shipping-late-and-bloated.</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Cuts scope decisively when timelines slip - protects the outcome-critical path, defers the rest, and tells affected stakeholders before they find out. Scope: their product area's releases.</t>
+          <t>Depth: Breaks own tasks into reviewable pieces with guidance. Evidenced by: Breaks their feature into reviewable pieces with a lead's guidance, and writes down what's lost if the last piece has to be cut. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Negotiates three-way trade-offs (scope, time, quality) with engineering as a peer, distinguishing an MVP that tests the hypothesis from a demo that fakes it, and refusing quality cuts that mortgage the roadmap. Scope: their product; engineering leads seek their trade-off call rather than working around them.</t>
+          <t>Depth: Independently decomposes a feature into shippable slices. Evidenced by: Cuts a feature's scope decisively when the sprint slips, protects the outcome-critical path, and tells the affected stakeholder before they notice on their own. Scope: a product area.</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Untangles trade-offs that span teams - where one area's cut breaks another's launch - and sets the shared definition of "minimum" for cross-area releases. Scope: multiple product areas.</t>
+          <t>Depth: Plans complex multi-phase work (prototype-then-commit under uncertainty); sequences safely. Evidenced by: Negotiates a scope-versus-quality trade-off with engineering as a peer, distinguishing an MVP that genuinely tests the hypothesis from a demo that only fakes it. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org's norms for scope discipline - MVP standards, quality floors, cut-decision authority - and intervenes when a flagship effort is bloating toward a death march. Scope: product org.</t>
+          <t>Depth: Expert at structuring large initiatives to de-risk early; anticipates bottlenecks. Evidenced by: Sets the shared definition of 'minimum' for a launch that spans three teams, untangling a scope disagreement that would otherwise have broken one team's release. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes the company-level calls on scope of ambition - when to ship the narrow wedge versus the platform play - in bets the whole portfolio sequences around. Scope: company portfolio.</t>
+          <t>Depth: Shapes how the org plans and sequences major change. Evidenced by: Sets the org's quality floor and cut-decision authority, and personally intervenes when a flagship initiative is bloating toward a death march. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines the company-wide approach to delivering value incrementally. Evidenced by: Makes the company-level call to ship the narrow wedge instead of the full platform play, and the rest of the portfolio sequences its bets around that decision. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -1989,37 +2100,42 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Cagan, *Empowered* (2020)</t>
+          <t>Works productively with others toward shared goals.</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Brings problems and evidence to engineers and designers early - not finished specs - and incorporates their feasibility and usability pushback into the plan visibly. Scope: one feature team.</t>
+          <t>Cagan &amp; Jones, EMPOWERED: Ordinary People, Extraordinary Products (Wiley, 2020) — empowered product teams of PM, design, and engineering solving problems together, versus feature teams served requirements; the PM-engineering-design relationship is the production function.</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs a working trio: engineers join discovery calls, designers see strategy context, and technical constraints reshape the product approach rather than getting escalated as blockers. Scope: their product area's team.</t>
+          <t>Depth: Responsive to feedback; pairs willingly; asks for help appropriately. Evidenced by: Takes feedback from an engineer's pushback on a spec without defensiveness, and asks the designer for help scoping a problem instead of guessing alone. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds a team engineers and designers ask to join - shares full business context, defends the team's discovery time, creates the safety for the best idea to win regardless of whose it was, observably in decision records. Scope: their product; their trio is cited internally as how it should work.</t>
+          <t>Depth: Collaborates smoothly with adjacent functions; handles disagreement constructively. Evidenced by: Runs a working trio where the engineer joins discovery calls and the designer sees the strategy context, so a technical constraint reshapes the plan in the room instead of becoming a later escalation. Scope: a product area.</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Repairs dysfunctional PM-engineering-design relationships on other teams, diagnosing whether the failure is context-starvation, requirement-throwing, or trust, and coaching the fix. Scope: multiple product areas.</t>
+          <t>Depth: Builds strong cross-team relationships; resolves friction directly. Evidenced by: Builds a team that engineers ask to be assigned to, sharing full business context and visibly deferring to the best idea in a decision record regardless of whose it was. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes the org's team model - how trios form, what empowerment means operationally, how tech-debt time is protected - in norms engineering and design leadership co-sign. Scope: product org.</t>
+          <t>Depth: Expert at aligning teams with competing priorities; mediates disputes between senior people. Evidenced by: Diagnoses that a struggling team's dysfunction is context-starvation rather than a trust problem, and coaches the PM through fixing it. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the company's bar for how product, engineering, and design work together, arguing the empowered-team model at the executive level when delivery pressure pushes toward feature factories. Scope: company portfolio.</t>
+          <t>Depth: Creates the forums and processes through which collaboration happens. Evidenced by: Shapes the org's team model — how trios form, how tech-debt time gets protected — in norms engineering and design leadership both sign off on. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Builds coalitions at company scale and externally. Evidenced by: Argues the empowered-team model at the executive level when delivery pressure is pushing the org toward feature factories, and the model holds. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2046,37 +2162,42 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Bryar &amp; Carr, *Working Backwards* (2021)</t>
+          <t>Translating problems into clear, testable requirements, specs, and acceptance criteria.</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes user stories with acceptance criteria that engineers implement without re-asking the basics, and keeps the spec updated as decisions land. Scope: one epic's spec.</t>
+          <t>IIBA, A Guide to the Business Analysis Body of Knowledge (BABOK Guide), Version 3 (2015) — substituted for Bryar &amp; Carr's Working Backwards (no bibliography entry) with BABOK, the requirements body of knowledge PM-07's own P2 catalog level already cites, paired with ISO/IEC/IEEE 29148's requirement-quality characteristics at P3 (unambiguous, verifiable, necessary).</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes one-pagers and PRDs that lead with the customer problem and success measures, covering edge cases and non-goals; the build raises design questions, not intent questions. Scope: their area's definition docs.</t>
+          <t>Depth: Writes requirements from supplied input and refines them under review. Evidenced by: Writes user stories with acceptance criteria from a lead's outline, and updates the spec twice as review catches gaps in the edge cases. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes specs that de-risk before build - working-backwards narratives whose FAQ answers the hard questions first - and their review comments on others' specs prevent rework. Scope: a product; their spec format is the team standard.</t>
+          <t>Depth: Authors complete, testable specs for standard features with normal review. Evidenced by: Writes a one-pager that leads with the customer problem and success measure for a standard feature, and the build raises design questions rather than intent questions. Scope: a product area.</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets definition standards across teams and reviews cross-team specs for interface gaps - the places where two teams' documents silently disagree. Scope: multiple product areas.</t>
+          <t>Depth: Independently specifies ambiguous, cross-cutting features and resolves edge cases cleanly. Evidenced by: Specifies a cross-cutting feature touching three systems, resolving edge cases the initial ask never anticipated, and a reviewer's comments on the spec prevent a rework two weeks later. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns the org's definition bar - what "ready to build" means org-wide - and their document reviews are the org's quality gate for major initiatives. Scope: product org.</t>
+          <t>Depth: Defines specification standards others adopt and untangles the hardest requirement conflicts. Evidenced by: Sets the definition-of-ready standard two other teams adopt, and catches an interface gap between two teams' specs that would have silently conflicted at integration. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes the founding documents for portfolio bets - the PR/FAQ or narrative that greenlights a new product line - with a hit rate the company trusts. Scope: company portfolio.</t>
+          <t>Depth: Sets specification strategy across teams and anticipates downstream definition needs. Evidenced by: Owns what 'ready to build' means across the product org, and their document review is the quality gate a major initiative has to pass before engineering starts. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what excellent product specification means and influences the practice externally. Evidenced by: Writes the founding narrative document for a new portfolio bet, with a hit rate on greenlit narratives the company has come to trust. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2103,37 +2224,42 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Patton, *User Story Mapping* (2014); Reinertsen, *The Principles of Product Development Flow* (2009)</t>
+          <t>Curating, refining, and grooming a backlog so the team always works on the highest-value items.</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps their epic's stories small, ordered, and ready two sprints ahead, and answers "what's next and why" without opening the tool. Scope: one epic's backlog.</t>
+          <t>Patton, User Story Mapping: Discover the Whole Story, Build the Right Product (O'Reilly, 2014) — story maps preserve the big picture a flat backlog destroys, paired with Reinertsen's small-batches and limited-WIP flow principles.</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Maintains a story map that shows the release strategy at a glance, slices releases thin, runs the team's planning rituals cleanly, and watches WIP and cycle time with the team. Scope: their area's delivery flow.</t>
+          <t>Depth: Updates and grooms backlog items under direction. Evidenced by: Keeps their epic's stories small, ordered, and ready two sprints ahead, and can answer 'what's next and why' without opening the tracking tool. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Diagnoses delivery problems from flow data - batch size, queue buildup, aging WIP - and fixes the system rather than pushing the team; their story maps anchor multi-quarter plans. Scope: a product's delivery system; other PMs copy their mapping sessions.</t>
+          <t>Depth: Prioritizes and maintains a healthy backlog for one team with normal review. Evidenced by: Maintains a story map that shows their area's release strategy at a glance, and watches WIP and cycle time with the team without waiting for someone else to flag a problem. Scope: a product area.</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Untangles cross-team delivery dependencies - shared components, sequencing, integration risk - before they surface as slips. Scope: multiple product areas.</t>
+          <t>Depth: Independently sequences contested work and keeps the backlog coherent under churn. Evidenced by: Diagnoses that a team's slipping deadlines are a queue-buildup problem, not a motivation problem, and fixes the batch size rather than pushing the team to work harder. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Improves the org's end-to-end flow - the idea-to-live lead time - by changing planning and handoff mechanics, with before/after numbers. Scope: product org.</t>
+          <t>Depth: Defines backlog practices others follow and resolves cross-team prioritization disputes. Evidenced by: Resolves a cross-team prioritization dispute using a shared backlog-sequencing standard other PMs have adopted from their earlier work. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Removes company-scale delivery drag - the portfolio-level process, tooling, or structure that slows every team - with executive backing they built. Scope: company portfolio.</t>
+          <t>Depth: Sets backlog-management strategy across products and anticipates capacity tensions. Evidenced by: Improves the org's idea-to-live lead time by changing planning and handoff mechanics, with before-and-after numbers to show it. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines backlog-management best practice for the discipline and is recognized for it. Evidenced by: Removes a company-scale delivery bottleneck — a shared review gate every team was queuing behind — with executive backing they built the case for. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2160,37 +2286,42 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Cagan, *Inspired* (2nd ed., 2018)</t>
+          <t>Retains enough hands-on technical depth to earn engineers' trust, ask the questions that change designs, and judge technical work without doing it.</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Follows the team's technical discussions and asks clarifying questions that show the homework was done - understands the platform's basic architecture and can tell deliberate design from decoration. Scope: one epic's technical and design context.</t>
+          <t>Cagan, INSPIRED: How to Create Tech Products Customers Love, 2nd Edition (Wiley, 2018) — deep knowledge of the technology and of good design is part of the PM's non-delegable preparation; a PM who can't follow the architecture or judge a design hands the feasibility and usability risks to whoever speaks last.</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands the architecture and dependencies of their area well enough to anticipate implementation challenges - raises security, scalability, and migration questions before engineers have to, and gives design feedback designers act on. Scope: their product area's stack and surfaces.</t>
+          <t>Depth: Follows the team's technical discussions and asks clarifying questions; relies on others to evaluate design quality. Evidenced by: Follows the team's architecture discussion and asks a clarifying question that shows they did the reading, deferring to the engineers on which design is better. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Holds their own in architecture and design trade-off discussions - understands the cost drivers and constraints of the systems their product rides on, spots when a proposed solution fights the architecture, and dogfoods builds critically. Scope: their product; engineers bring them options early because the conversation is worth it.</t>
+          <t>Depth: Understands the systems in scope well enough to review designs, probe trade-offs, and triage incidents — earns technical respect without taking the keyboard. Evidenced by: Reviews a proposed design well enough to raise a scalability question before an engineer has to, and triages a live incident credibly without touching the code. Scope: a product area.</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Bridges technical constraints across teams - catches when one area's roadmap assumes capabilities another team's architecture can't deliver, and translates platform trade-offs into product terms for other PMs. Scope: multiple product areas.</t>
+          <t>Depth: Maintains depth across a complex system's stack and hardest problems; a credible thought-partner to the most senior engineers, pairing them with the context they need. Evidenced by: Holds their own in an architecture trade-off discussion, spotting that a proposed solution fights the existing system before the team commits to it, and engineers bring them options early because the conversation is worth it. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps the org's product decisions technically honest - represents platform realities in org planning and raises other PMs' technical fluency through review and teaching. Scope: product org.</t>
+          <t>Depth: Maintains depth across a complex system's stack and hardest problems; a credible thought-partner to the most senior engineers, pairing them with the context they need. Evidenced by: Bridges a technical constraint between two teams' roadmaps that neither team's own engineers had connected, translating the platform trade-off into terms the other PM can act on. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Frames company-level technology inflections in product terms - platform shifts, build/buy - reliably enough that executives act on the translation, while deferring deep technical authority to engineering leaders. Scope: company portfolio.</t>
+          <t>Depth: Retains broad credibility across a multi-team domain — credible on its hardest cross-cutting technical questions, current enough to ask the question that changes a design. Evidenced by: Keeps the product org's planning technically honest by representing platform realities in a strategy review, deferring the deepest technical call to the engineering leader in the room. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Retains broad credibility across a multi-team domain — credible on its hardest cross-cutting technical questions, current enough to ask the question that changes a design. Evidenced by: Frames a company-level build-versus-buy technology inflection in product terms clearly enough that executives act on the translation, while the technical authority for the decision itself stays with engineering leadership. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2217,37 +2348,42 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Cagan, *Inspired* (2nd ed., 2018)</t>
+          <t>Orchestrating launch readiness across engineering, marketing, sales, and support.</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs the launch checklist for their feature - flags, docs, support notes, comms - and staffs the first-day triage, escalating what they can't resolve. Scope: one feature launch.</t>
+          <t>Cagan, INSPIRED: How to Create Tech Products Customers Love, 2nd Edition (Wiley, 2018) — high-integrity commitments and launch readiness across the whole company, not just the code, paired with Kohavi et al.'s ramped-rollout-and-holdback pattern as the safe launch mechanism.</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Plans and runs launches for their area end-to-end: rollout stages, success/rollback criteria decided in advance, and every dependent function briefed before go-live. Scope: their product area's launches.</t>
+          <t>Depth: Executes assigned launch tasks and tracks checklist items under guidance. Evidenced by: Runs the launch checklist for their feature — flags, docs, support notes — and staffs first-day triage, escalating what they can't resolve to their lead. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns launch calls under pressure - go/no-go, ramp pace, rollback - with criteria set before emotions run, and runs the post-launch review that feeds the next iteration. Scope: their product; other teams copy their launch-readiness template.</t>
+          <t>Depth: Coordinates a standard product launch across functions with normal review. Evidenced by: Plans a standard launch end to end: rollout stages and rollback criteria decided in advance, every dependent function briefed before go-live. Scope: a product area.</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Coordinates launches that span teams and products, sequencing dependencies and owning the integrated go/no-go where no single team can. Scope: multiple product areas.</t>
+          <t>Depth: Independently orchestrates complex launches and recovers when plans go sideways. Evidenced by: Makes the go/no-go call on a ramping launch under pressure using criteria set the week before, not in the moment, and runs the post-launch review that feeds the next iteration. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org's launch discipline - readiness standards, ramp policy, review practice - and is the escalation point for the launches with company-level blast radius. Scope: product org.</t>
+          <t>Depth: Defines the go-to-market playbook others adopt and rescues high-stakes launches. Evidenced by: Owns the integrated go/no-go for a launch spanning three teams' products, sequencing each team's dependency so no single team's slip silently blocks the others. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns company-defining launches - the ones with board visibility and market coverage - and sets the standard for what the company considers launch-ready. Scope: company portfolio.</t>
+          <t>Depth: Sets go-to-market strategy across the portfolio and anticipates market-timing risks. Evidenced by: Sets the org's ramp-policy and readiness standards, and is the escalation point when a launch with company-level blast radius needs a call above any one team. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what great go-to-market means for the field and shapes external practice. Evidenced by: Owns the go/no-go for a launch with company-wide stakes as a high-integrity commitment the whole company is briefed on, not just engineering. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2274,37 +2410,42 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Olsen, *The Lean Product Playbook* (2015)</t>
+          <t>Defining success metrics and interpreting product data to evaluate impact and guide iteration.</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Tracks their feature's post-launch metrics against the targets set pre-launch and reports the gap honestly, proposing the first follow-up fix. Scope: one feature's first iterations.</t>
+          <t>Croll &amp; Yoskovitz, Lean Analytics: Use Data to Build a Better Startup Faster (O'Reilly, 2013) — substituted for Olsen's The Lean Product Playbook (no bibliography entry) with Croll &amp; Yoskovitz's stage-based Lean Analytics Cycle — empathy, stickiness, virality, revenue, scale — which is the same anchor family PM-10's other rows above use and covers persevere/pivot/kill judgment directly.</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Budgets iteration capacity into every launch plan and runs the loop - measure, diagnose, fix, re-measure - until the feature hits its outcome or is deliberately parked. Scope: their product area.</t>
+          <t>Depth: Pulls and reports defined product metrics under direction. Evidenced by: Reports their feature's week-one usage numbers exactly as their lead asked, without yet proposing what the team should do differently. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes the persevere/pivot/kill call on their product's bets on the evidence rather than sunk cost, and sunsets features with a migration plan, resisting the portfolio-of-zombies default. Scope: their product; the deprecation they ran is the template others use.</t>
+          <t>Depth: Builds and interprets metric dashboards for a product with normal review. Evidenced by: Reads a newly-launched feature's numbers against the product's current lifecycle stage and proposes the next iteration to try before the next planning cycle. Scope: a product area.</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Audits post-launch follow-through across teams, surfacing launched-and-abandoned features and getting iteration capacity re-protected. Scope: multiple product areas.</t>
+          <t>Depth: Independently designs metric frameworks and draws sound conclusions from messy data. Evidenced by: Makes the persevere-pivot-kill call on a six-month-old feature using its own metric framework, and the recommendation holds up under a skeptical leadership review. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Manages lifecycle at org level - which products get investment, maintenance, or end-of-life - with criteria applied consistently enough that teams predict the outcome. Scope: product org.</t>
+          <t>Depth: Defines the measurement model teams adopt and diagnoses misleading metrics others trust. Evidenced by: Diagnoses that a metric two other teams trust as a success signal is actually misleading at this lifecycle stage, and gets both teams onto a corrected measurement model. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Makes the company's hardest lifecycle calls - killing revenue-bearing products, betting through the J-curve - with reasoning the executive team adopts. Scope: company portfolio.</t>
+          <t>Depth: Sets product-analytics strategy across the org and anticipates which signals will matter. Evidenced by: Sets the analytics strategy for what 'iterating well post-launch' means across the whole product org, anticipating which signals will matter before a product reaches that stage. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines rigorous product measurement for the discipline and is cited externally on it. Evidenced by: Defines a measurement discipline for post-launch iteration that gets cited by other companies as a rigorous approach to persevere/pivot/kill decisions. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2331,37 +2472,42 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Osterwalder &amp; Pigneur, *Business Model Generation* (2010)</t>
+          <t>Frames technical decisions in economic and business terms — cost, revenue risk, cost of delay, unit economics — and answers for whether the work actually moved its business outcome.</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Explains how their product makes money - who pays, for what, through which motion - and traces how their feature touches cost or revenue, with coaching. Scope: one feature's business context.</t>
+          <t>Osterwalder &amp; Pigneur, Business Model Generation (Wiley, 2010) — the Business Model Canvas's nine building blocks are the standard template for reasoning about how a product actually sustains itself economically.</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds simple business cases for their area's bets - revenue or cost impact, rough unit economics - and sanity-checks them with finance before pitching. Scope: their product area.</t>
+          <t>Depth: States what business outcome their current task serves — and asks when they can't — treating infrastructure and license costs as real money. Evidenced by: States which business outcome their current task serves when a lead asks, and flags that a chosen third-party tool carries a real per-seat license cost, not just an engineering cost. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns the viability case for their product: models how bets affect margin, CAC/LTV, or retention economics, and kills their own proposals when the economics don't clear. Scope: their product; finance treats their models as credible inputs.</t>
+          <t>Depth: Checks whether shipped work actually moved its metric and says so plainly when it didn't; weighs cost and maintenance burden in the technical choices they own. Evidenced by: Checks whether a feature shipped last quarter actually moved its target metric, and says plainly in the retro that it didn't, rather than letting the shipped-it framing stand. Scope: a product area.</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Pressure-tests business cases across teams, catching double-counted revenue and hockey-stick assumptions before they reach leadership. Scope: multiple product areas.</t>
+          <t>Depth: Frames a domain's technical decisions in business terms — cost of delay, revenue risk, support load — pushes back on work with weak business rationale, and redirects effort when the numbers say the plan is wrong. Evidenced by: Redirects a team's roadmap away from a planned initiative once cost-of-delay and support-load numbers show a cheaper, faster path serves the same outcome. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Connects the org's product strategy to the P&amp;L - which products drive growth versus margin - in analyses the business planning cycle runs on. Scope: product org.</t>
+          <t>Depth: Builds the business case for the cross-team technical investments with the largest return and is trusted by leadership to have done the math. Evidenced by: Builds the business case for a cross-team platform investment with the largest expected return, and leadership funds it on the strength of the math. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes the company's business model evolution - monetization shifts, platform economics, new revenue lines - at the level the CFO and CEO debate. Scope: company portfolio.</t>
+          <t>Depth: Aligns an organization's technical strategy with its economics — cost curves, velocity, risk — owning trade-offs measured in staff-years and reporting them in the business's own terms. Evidenced by: Aligns the org's technical investment strategy with its cost curve and velocity trends, owning a trade-off measured in staff-years that leadership signs off on. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Advises company leadership on where technology changes the business model and is accountable for company-level technology bets paying off. Evidenced by: Advises company leadership on where a technology shift changes the business model itself, and is held accountable for whether the resulting company-level bet pays off. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2388,37 +2534,42 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Ramanujam &amp; Tacke, *Monetizing Innovation* (2016)</t>
+          <t>Reasoning about pricing, packaging, and unit economics to sustain a viable product.</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Knows their product's pricing and can state which plan gates their feature, and flags when a build decision would leak paid value into free. Scope: one feature's packaging context.</t>
+          <t>Nagle, Muller &amp; Gruyaert, The Strategy and Tactics of Pricing: A Guide to Growing More Profitably, 7th Edition (Routledge, 2023) — substituted for Ramanujam &amp; Tacke's Monetizing Innovation (no bibliography entry) with Nagle, Muller &amp; Gruyaert's value-based pricing text, PM-12's own catalog anchor for the P3/P4/P6 levels — the value cascade against cost-plus defaults.</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Raises willingness-to-pay questions during discovery, bringing upgrade/downgrade and win/loss signals into roadmap discussions, and flags when a feature belongs in a different tier than assumed. Scope: their product area's packaging fit.</t>
+          <t>Depth: Populates pricing models with supplied assumptions under direction. Evidenced by: Fills in a pricing model with the cost and margin assumptions a lead supplied, and asks when an input looks wrong rather than silently accepting it. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives a pricing or packaging change for their product - research, value-metric modeling, migration plan - in partnership with pricing owners as a peer. Scope: a product's monetization; pricing changes in their area don't happen without them in the room.</t>
+          <t>Depth: Builds a sound business model for one product with normal review. Evidenced by: Builds the revenue-stream section of a new feature's business model using the team's standard canvas, and it holds up under normal review. Scope: a product area.</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Resolves packaging conflicts between products (bundling, gating, tier coherence) so the catalog makes sense to buyers, and reviews new packaging for cannibalization. Scope: multiple product areas.</t>
+          <t>Depth: Independently structures pricing under uncertainty and defends margin trade-offs. Evidenced by: Defends a value-based price increase to a skeptical sales leader with a margin trade-off argument, instead of defaulting to a cost-plus number that's easier to justify. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes the org's monetization strategy - pricing metric, tier architecture, discount posture - with research and modeling leadership funds decisions from. Scope: product org.</t>
+          <t>Depth: Defines the modeling approach others adopt and untangles complex monetization questions. Evidenced by: Defines the pricing-modeling approach two other product teams adopt, and untangles a monetization question — a bundling decision with conflicting margin implications — no single team's model could resolve. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets company-level pricing philosophy - how the company captures the value it creates - in frameworks that persist across individual pricing decisions. Scope: company portfolio.</t>
+          <t>Depth: Sets pricing strategy across the portfolio and anticipates market and cost shifts. Evidenced by: Sets the portfolio's pricing strategy for the year, anticipating a cost shift in a key input before it forces a reactive repricing. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines pricing and business-modeling best practice for the field and is recognized for it. Evidenced by: Defines a pricing and business-modeling practice recognized in the field, with other companies' pricing teams citing the approach. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2445,37 +2596,42 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Moore, *Crossing the Chasm* (3rd ed., 2014)</t>
+          <t>Assessing market trends, competitors, and whitespace to inform positioning and opportunity sizing.</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Produces a current, accurate comparison of how named competitors solve their feature's problem, from hands-on use of the competitor products where possible. Scope: one feature's competitive slice.</t>
+          <t>Moore, Crossing the Chasm: Marketing and Selling High-Tech Products to Mainstream Customers, 3rd Edition (HarperBusiness, 2014; orig. 1991) — the technology-adoption-lifecycle model and the chasm between early adopters and the mainstream market require reading ambiguous markets, not just cataloging named competitors.</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Maintains a living competitive view for their area - releases tracked, win/loss notes read, sales anecdotes verified against evidence - and separates competitor moves worth responding to from noise. Scope: their product area.</t>
+          <t>Depth: Gathers competitor facts and populates comparison grids under guidance. Evidenced by: Populates a competitive comparison grid with facts a lead asked them to gather, and gets it corrected twice on review before it's accurate. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Reads the market structurally for their product - substitutes, adjacent entrants, disruption vectors, not just feature parity - and their competitive assessments visibly shape the strategy doc. Scope: their product; sales asks them for the competitive narrative, not the reverse.</t>
+          <t>Depth: Produces a sound competitive analysis for a product with normal review. Evidenced by: Produces a competitive analysis for their product using the team's standard framework, and it holds up without a rewrite in the next planning cycle. Scope: a product area.</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Synthesizes market intelligence across areas into portfolio-level threat and opportunity calls other PMs plan against. Scope: multiple product areas.</t>
+          <t>Depth: Independently reads ambiguous markets and frames defensible positioning implications. Evidenced by: Reads an ambiguous, fragmenting market correctly enough to argue the product hasn't crossed the chasm yet, and rewrites their product's positioning to match before the next release. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns the org's market thesis - where the market is going and how the org wins there - updated on evidence and defended in planning. Scope: product org.</t>
+          <t>Depth: Defines the analytical approach others follow and decodes confusing competitive dynamics. Evidenced by: Defines the competitive-analysis method two other product teams adopt, and decodes a confusing competitive move — a rival's pricing change that looked irrational — that had stumped both teams. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Anticipates industry shifts at company level - platform transitions, business-model disruptions - early enough for the portfolio to reposition, in analyses the board sees. Scope: company portfolio.</t>
+          <t>Depth: Sets market-analysis strategy and anticipates structural shifts before competitors react. Evidenced by: Anticipates a structural market shift a full product cycle before competitors react to it, and repositions the portfolio's investment ahead of the shift. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes how the field interprets product-market fit and is cited externally on it. Evidenced by: Shapes how the field talks about product-market fit in this category, cited by analysts and competitors alike. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2502,37 +2658,42 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Cagan, *Inspired* (2nd ed., 2018)</t>
+          <t>Builds and maintains deep working knowledge of the product's domain — its industry structure, customer workflows, constraints, and trajectory — deeply enough to be a credible reference for customers and colleagues.</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Learns the domain deliberately - shadows customers, reads the industry sources, asks engineers how the system actually works - and stops needing the glossary. Scope: their epic's domain slice.</t>
+          <t>Cagan, INSPIRED: How to Create Tech Products Customers Love, 2nd Edition (Wiley, 2018) — deep, non-delegable knowledge of the customer, business, and industry domain; self-sourced capability (PM-19 minted 2026-07 from this ladder's own prior consolidation prose — see scope_note), so evidence is written fresh below.</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Answers most domain questions in refinement without deferring, corrects domain errors in specs and designs, and understands the operational challenges of the products they run. Scope: their product area's domain.</t>
+          <t>Depth: Learns the domain deliberately — shadows customers, reads industry sources, asks how the system actually works — and uses domain vocabulary correctly. Evidenced by: Shadows a customer support call and reads the industry's standard reference material, and uses the domain's own vocabulary correctly in their first spec review. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Is the recognized domain reference for their product - customers, field teams, and engineers check facts with them - and spots domain-driven risks others miss. Scope: a product's domain.</t>
+          <t>Depth: Answers most domain questions without deferring and corrects domain errors in specs and designs. Evidenced by: Answers a stakeholder's domain question about a regulatory constraint without deferring to a subject-matter expert, and corrects a domain error in an engineer's design before it ships. Scope: a product area.</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Connects domain knowledge across areas, catching where one team's roadmap violates another domain's constraints (regulatory, workflow, ecosystem). Scope: multiple product areas.</t>
+          <t>Depth: Is the recognized domain reference for a product — customers, field teams, and engineers check facts with them — and spots domain-driven risks others miss. Evidenced by: Becomes the person the field team calls to fact-check a claim about how the industry's workflow actually works, and spots a domain-driven risk in a proposed feature nobody else caught. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Represents the company's domain understanding externally - industry forums, customer advisory boards, analyst briefings. Scope: product org.</t>
+          <t>Depth: Connects domain knowledge across teams, catching where one roadmap violates another domain's constraints (regulatory, workflow, ecosystem). Evidenced by: Catches that one team's roadmap assumes a regulatory workflow another team's domain constraints actually forbid, before either team ships something that has to be walked back. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Anticipates domain evolution - where the industry's workflows and rules are heading - and seeds the portfolio for it. Scope: company portfolio.</t>
+          <t>Depth: Represents an organization's domain understanding externally — industry forums, advisory boards, analyst briefings. Evidenced by: Represents the org's domain understanding on an industry advisory board, bringing back a signal the org's roadmap hadn't accounted for. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Anticipates domain evolution — where the industry's workflows and rules are heading — and positions portfolios for it before consensus forms. Evidenced by: Positions the portfolio ahead of a domain shift — a regulatory change on the horizon — before industry consensus has formed that it's coming. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2559,37 +2720,42 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Moore, *Crossing the Chasm* (3rd ed., 2014)</t>
+          <t>Orchestrating launch readiness across engineering, marketing, sales, and support.</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Delivers accurate launch inputs to GTM teams - what changed, who it's for, what to say - on their timeline, using the team's launch template. Scope: their feature's GTM inputs.</t>
+          <t>Moore, Crossing the Chasm: Marketing and Selling High-Tech Products to Mainstream Customers, 3rd Edition (HarperBusiness, 2014; orig. 1991) — adoption is won segment by segment; a launch that doesn't land in its intended beachhead segment needs Moore's chasm-crossing recovery logic, not a bigger push.</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs launch readiness for their area with marketing, sales, and support - tiering the launch, agreeing the bill of materials, confirming enablement landed before GA. Scope: a product area's launches.</t>
+          <t>Depth: Executes assigned launch tasks and tracks checklist items under guidance. Evidenced by: Executes their assigned launch-day tasks from the GTM checklist and escalates a customer-support question they can't answer to the person who can. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Plans GTM as part of product strategy, not an afterthought - segment-specific whole-product gaps identified in discovery, channel fit argued in the spec; GTM partners treat them as a peer planner. Scope: a product's route to market.</t>
+          <t>Depth: Coordinates a standard product launch across functions with normal review. Evidenced by: Coordinates a standard launch across sales, marketing, and support using the team's established playbook, with every function briefed before go-live. Scope: a product area.</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Aligns GTM motions across products sold together - shared plays, coherent bundles, one story to the same buyer. Scope: multiple product areas.</t>
+          <t>Depth: Independently orchestrates complex launches and recovers when plans go sideways. Evidenced by: Recovers a launch that isn't landing in its intended beachhead segment by re-targeting mid-rollout instead of pushing harder on a segment that isn't buying. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes the org's GTM model jointly with sales and marketing leadership - PLG vs. sales-led boundaries, launch tiering standards, readiness gates. Scope: product org.</t>
+          <t>Depth: Defines the go-to-market playbook others adopt and rescues high-stakes launches. Evidenced by: Defines the go-to-market playbook two other product teams now use, and personally rescues a launch that had gone sideways days before its public date. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Architects company-level GTM shifts - new channels, new buyer motions - tied to portfolio strategy and carried through executive planning. Scope: company portfolio.</t>
+          <t>Depth: Sets go-to-market strategy across the portfolio and anticipates market-timing risks. Evidenced by: Sets go-to-market strategy across the portfolio, timing two products' launches to avoid cannibalizing each other's market attention. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what great go-to-market means for the field and shapes external practice. Evidenced by: Shapes what great go-to-market means for the field, with the launch approach cited by practitioners outside the company. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2616,37 +2782,42 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Cagan, *Inspired* (2nd ed., 2018)</t>
+          <t>Building trust with customers and external partners to inform and advance the product.</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Works support tickets and sales notes for their feature into the backlog with the underlying problem stated, not the ticket verbatim. Scope: their feature's field signal.</t>
+          <t>Cagan, INSPIRED: How to Create Tech Products Customers Love, 2nd Edition (Wiley, 2018) — field and customer-facing teams are a product's highest-bandwidth feedback channel and the most direct enablement surface — closing that loop is part of the PM's non-delegable work, not a hand-off to enablement.</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs a regular loop with sales and support for their area - win/loss notes, top-ticket themes, deal-blocker reviews - and closes the loop by telling the field what shipped because of them. Scope: a product area's feedback system.</t>
+          <t>Depth: Logs interactions and handles routine customer requests under guidance. Evidenced by: Logs a field team's escalated customer request in the team's tracker and hands off routine ones using the process a lead set up. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Filters field pressure into strategy without being captured by it - separates the loudest deal from the pattern, says no to one-off asks in writing, and maintains reference customers who co-develop. Scope: a product's field relationship; sales leadership trusts their no.</t>
+          <t>Depth: Manages standard customer and partner relationships with normal review. Evidenced by: Runs the monthly loop that turns field-team feedback into a prioritized list their product area actually acts on, with normal review from a lead. Scope: a product area.</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds shared field-signal infrastructure across teams - one win/loss taxonomy, one escalation path - so patterns spanning products become visible. Scope: multiple product areas.</t>
+          <t>Depth: Independently nurtures key accounts and resolves difficult relationship conflicts. Evidenced by: Personally rescues a strained relationship with a key account after a rocky launch, and the account renews where the field team had expected a churn. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs the org's field-to-product operating loop - councils, SLAs on responses, evidence standards for deal-driven asks. Scope: product org.</t>
+          <t>Depth: Defines relationship-management practices others adopt and salvages strained partnerships. Evidenced by: Defines the field-enablement practice two other teams now use to close their own feedback loops, and salvages a partnership another team's process had let go stale. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps the company's biggest customer relationships strategically productive - executive briefing programs and co-innovation loops that inform portfolio bets without hijacking them. Scope: company portfolio.</t>
+          <t>Depth: Sets relationship strategy across the portfolio and anticipates partner-ecosystem shifts. Evidenced by: Sets partner-ecosystem strategy across the portfolio, anticipating a shift in a key partner's priorities before it disrupts a live integration. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what excellent partner relationship management means and shapes external practice. Evidenced by: Defines what excellent partner relationship management looks like for the discipline, in practice other companies' product teams point to. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2673,37 +2844,42 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Bryar &amp; Carr, *Working Backwards* (2021)</t>
+          <t>Conveys ideas clearly to the right audience.</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes clear, structured updates and one-pagers - one idea per paragraph, conclusion visible early - that readers act on without a follow-up meeting. Scope: their epic's documents.</t>
+          <t>Zinsser, On Writing Well: The Classic Guide to Writing Nonfiction, 30th Anniversary Edition (Harper Perennial, 2006) — substituted for Bryar &amp; Carr's Working Backwards (no bibliography entry) with Zinsser's classic clarity-in-writing reference for the baseline register, paired with Minto's pyramid principle for the decision-driving register — the same two-source pairing CC-01's own catalog levels already use.</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes narratives that carry decisions - the six-pager or one-pager that a review reads silently and then debates on substance, not on what the author meant. Scope: their area's decision documents.</t>
+          <t>Depth: Communicates status clearly; documentation is accurate. Evidenced by: Writes a status update for their epic that says plainly what happened and what's next, without burying the headline in caveats. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes documents that move people who weren't in the room - strategy narratives forwarded beyond their audience, quoted in others' plans; their edits make colleagues' drafts decision-ready. Scope: a product; their documents are the team's writing exemplars.</t>
+          <t>Depth: Writes clear design notes, runbooks and PRs; explains trade-offs without overselling. Evidenced by: Writes a PRD for a standard feature that explains a trade-off honestly rather than overselling it, and engineers don't need to re-ask the intent. Scope: a product area.</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Raises writing quality across teams through review - narrative standards, document templates, and edit passes that measurably shorten decision cycles. Scope: multiple product areas.</t>
+          <t>Depth: Writes design docs that drive decisions; translates technical risk for non-technical stakeholders. Evidenced by: Writes a design doc that leads with the decision it's asking for and translates a technical risk into terms a non-technical stakeholder acts on correctly. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Authors the org's canonical documents - the strategy, the operating doc, the annual narrative - that stay accurate enough to be load-bearing. Scope: product org.</t>
+          <t>Depth: Expert at making complex capability/risk legible to executives without dumbing it down; RFCs align orgs. Evidenced by: Writes an RFC that aligns three teams' engineering leads on a shared approach, pre-wired against the objections a skeptic would raise. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes artifacts with company-level and external reach - vision papers, keynote narratives, published essays - that shape how the market and the company describe the strategy. Scope: company portfolio and industry.</t>
+          <t>Depth: Strategy memos leadership acts on; org-wide and external reach. Evidenced by: Writes a strategy memo that leadership funds a quarter's roadmap against, with reach beyond their own product organization. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Depth: A clarifying voice at company scale; externally recognized. Evidenced by: Is the clarifying voice the company turns to for its hardest external communications, recognized outside the company for writing that cuts through noise. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2730,37 +2906,42 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Minto, *The Pyramid Principle* (1987)</t>
+          <t>Communicates upward and to executive audiences — answer-first briefings, decision-ready framing, and composure under hostile questioning.</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Presents their epic's status in three sentences - situation, risk, ask - and answers executive follow-ups with data or an honest "I'll find out" rather than improvising. Scope: their epic in team-level reviews.</t>
+          <t>Minto, The Minto Pyramid Principle: Logic in Writing, Thinking, and Problem Solving (Minto International, 1996) — answer-first, decision-ready framing and composure under hostile questioning; paired with Grove's account of high-leverage management communication.</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs their own slot in leadership reviews: leads with the decision needed, anticipates the two hardest questions, and follows up in writing on every commitment made. Scope: their product area's reviews.</t>
+          <t>Depth: Prepares status updates for leadership with guidance; leads with the headline when coached to. Evidenced by: Prepares a status update for a leadership review with a lead's coaching to lead with the headline instead of the chronology. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Handles hostile or high-pressure executive sessions without ceding the evidence - corrects a senior leader's wrong premise respectfully in the room, and converts vague executive direction into concrete, confirmable decisions. Scope: their product; leadership asks for them by name when their area is on the agenda.</t>
+          <t>Depth: Reports upward answer-first with a specific ask; escalates early with options attached, so no surprise reaches leadership from someone else. Evidenced by: Reports upward with the ask stated first and two options attached, so no surprise reaches their VP from someone else first. Scope: a product area.</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Preps other PMs for executive moments - reviews their materials, red-teams the questions - and represents multi-team positions where no single PM has the full picture. Scope: multiple product areas.</t>
+          <t>Depth: Briefs senior leaders under pressure — facts, impact, options, and a recommendation inside the first two minutes; one-pagers get forwarded unedited. Evidenced by: Briefs a room of senior leaders under time pressure with facts, impact, options, and a recommendation inside the first two minutes, and the one-pager gets forwarded unedited. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Operates as a standing counterpart to the executive team, shaping how product information reaches them and pushing decision authority back down when executives grab it. Scope: product org.</t>
+          <t>Depth: Builds and lands investment cases with executive audiences — pre-wired with skeptics, sized in business terms, honest about risk; coaches others for executive rooms and runs the operating reviews an organization communicates through. Evidenced by: Builds an investment case pre-wired against a known skeptic's objections, sized in business terms, and coaches a junior PM through their first executive review. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Communicates for the company - board sessions, analyst briefings, keynote narratives - with the credibility that the message and the product reality match. Scope: company portfolio.</t>
+          <t>Depth: Operates the executive room as a peer — advances positions, absorbs hostile questioning without defensiveness, and changes the room's decision more often than not. Evidenced by: Operates an executive review as a peer, absorbs hostile questioning without getting defensive, and changes the room's decision. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Speaks for an organization's technical reality to boards, investors, and press; trusted with the messages that cannot be delegated, and organizational credibility survives the appearances. Evidenced by: Speaks for the company's technical reality to the board and press on a message that can't be delegated, and the company's credibility survives the appearance. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2787,37 +2968,42 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Cagan, *Empowered* (2020)</t>
+          <t>Aligning leadership and cross-functional stakeholders around product direction and trade-offs.</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Keeps their stakeholders current without being chased - status, risks, and changes communicated before anyone has to ask. Scope: their epic's stakeholders.</t>
+          <t>Cagan &amp; Jones, EMPOWERED: Ordinary People, Extraordinary Products (Wiley, 2020) — building executive trust and aligning cross-functional stakeholders around product direction is the empowered product leader's codified practice for building the trust an empowered team depends on.</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Maps their area's stakeholders and pre-wires decisions - the meeting confirms alignment built one-on-one beforehand; surprises are rare and owned fast. Scope: a product area's stakeholder set.</t>
+          <t>Depth: Prepares updates and gathers input for stakeholders under direction. Evidenced by: Gathers input from three stakeholders ahead of a review and drafts the update summary a lead then finalizes. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Aligns stakeholders with conflicting interests around decisions that hold - disagreements surfaced early, trade-offs written down, and re-litigation declined by pointing at the record. Scope: a product; executives name them as the PM whose commitments they trust.</t>
+          <t>Depth: Manages routine stakeholder relationships and communications with normal review. Evidenced by: Manages a routine monthly stakeholder update on their own, fielding questions without needing a lead to step in. Scope: a product area.</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Brokers alignment across organizational seams - between product areas, or between product and adjacent functions - where no one owns the whole decision. Scope: multiple product areas.</t>
+          <t>Depth: Independently aligns conflicting stakeholders and navigates tense executive conversations. Evidenced by: Navigates a tense conversation between two stakeholders with conflicting asks to a decision both accept, without damaging either relationship. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Maintains durable trust with the executive stakeholder set - the standing credibility that lets the org make bold moves without escalation storms. Scope: product org.</t>
+          <t>Depth: Defines stakeholder-engagement approaches others adopt and brokers the hardest alignment. Evidenced by: Defines the stakeholder-engagement approach two other PMs now follow, and brokers an alignment between two VPs that had stalled for a quarter. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Aligns board-level and cross-company stakeholders on portfolio direction, absorbing and resolving the conflicts that would otherwise fragment strategy. Scope: company portfolio.</t>
+          <t>Depth: Sets executive-engagement strategy and anticipates leadership concerns before they arise. Evidenced by: Sets executive-engagement strategy for the product org and raises a leadership concern in a briefing before the leader had to ask about it. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines exemplary stakeholder management for the discipline and is externally credible on it. Evidenced by: Is the reference other product leaders point to for exemplary stakeholder management, credible on it outside the company. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2844,37 +3030,42 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Perri, *Escaping the Build Trap* (2018)</t>
+          <t>Navigates conflict toward good decisions.</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Routes new requests through the team's intake instead of quietly absorbing them, and tells requesters what happens next. Scope: one epic's intake.</t>
+          <t>Perri, Escaping the Build Trap: How Effective Product Management Creates Real Value (O'Reilly, 2018) — saying no to weak requests and negotiating trade-offs in the open is what protects the team's outcome focus from becoming a feature-request queue.</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Declines requests with the reasoning attached - what it competes with, what evidence would reopen it - so a "no" informs rather than deflects. Scope: a product area.</t>
+          <t>Depth: Voices disagreement respectfully; disagrees-and-commits. Evidenced by: Disagrees with a stakeholder's proposed scope respectfully in a planning meeting, and commits fully to the team's final call once it's made. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Says no to powerful people and keeps the relationship - the exec whose pet feature was declined still sponsors the product - because the strategy behind the no is visible and consistent. Scope: a product's demand boundary.</t>
+          <t>Depth: Works through disagreement to a decision without damaging relationships. Evidenced by: Works a disagreement over priority with a peer PM through to a decision both can live with, without either relationship taking damage. Scope: a product area.</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Backs other PMs' hard nos - reinforcing the strategic rationale when a declined stakeholder shops the request elsewhere - and negotiates cross-team conflicts to a resolution both sides execute. Scope: multiple product areas.</t>
+          <t>Depth: Mediates technical disputes in their domain; finds the path that holds up. Evidenced by: Mediates a technical dispute between two senior engineers over an approach, and the path the team ends up on holds up three months later. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the org's intake and escalation norms so nos are consistent and appealable through one path, and the org visibly does fewer, bigger things. Scope: product org.</t>
+          <t>Depth: Resolves high-stakes disagreements between senior stakeholders across orgs. Evidenced by: Resolves a high-stakes disagreement between two VPs from different orgs over a shared roadmap, where the stakes and organizational distance had stalled prior attempts. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Declines whole categories of opportunity at company level - the market not entered - with reasoning the company can repeat. Scope: company portfolio.</t>
+          <t>Depth: Designs the decision processes the org uses to resolve conflict. Evidenced by: Designs the decision process the org now uses to resolve cross-team prioritization conflicts, replacing a pattern of escalations that used to land on one exec's desk. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Sets the company norm for principled disagreement. Evidenced by: Sets the company norm for how principled disagreement gets resolved, cited when new leaders are onboarded into how the company makes contested calls. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2901,37 +3092,42 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>Cagan, *Empowered* (2020)</t>
+          <t>Grows other people's capability.</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Seeks feedback concretely and applies it visibly - asks "what would you have done differently," and the next artifact shows the change; helps onboard newer peers with honest "what I wish I'd known" context. Scope: their own growth plus one peer at a time.</t>
+          <t>Cagan &amp; Jones, EMPOWERED: Ordinary People, Extraordinary Products (Wiley, 2020) — growing other PMs' capability compounds a product organization's craft beyond any one person's individual output.</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Mentors an APM or new PM on real work - reviews their docs before meetings, debriefs their calls - improving the mentee's output measurably without doing it for them. Scope: one or two mentees in their orbit.</t>
+          <t>Depth: Receptive to mentoring; shares what they learn. Evidenced by: Takes a senior PM's feedback on a spec without defensiveness and passes the lesson along to a newer teammate a week later. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Develops the PMs around them as a working habit - structured feedback on strategy docs, shared interview reps, honest gap conversations - and mentees can name specific skills they got from this person. Scope: PMs on and adjacent to their product; a recognized mentor without any reporting line.</t>
+          <t>Depth: Helps onboard teammates; informally mentors juniors. Evidenced by: Helps a new PM get their first feature shipped by walking them through the team's discovery cadence, without being formally assigned as their mentor. Scope: a product area.</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs deliberate craft development across teams - coaching plans, skill assessments, PM community sessions - and managers route struggling PMs to them for craft coaching. Scope: multiple product areas' PM population.</t>
+          <t>Depth: Coaches engineers with growth-oriented feedback; measurably improves a team's skill. Evidenced by: Coaches a struggling PM through three consecutive cycles of feedback that visibly improves their spec-writing, measured in fewer clarifying questions from engineering. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the org's PM development system - competency expectations, onboarding curriculum, senior-PM readiness bar - and personally develops the next generation of craft leaders. Scope: product org.</t>
+          <t>Depth: Develops future leads across teams; shapes hiring and onboarding. Evidenced by: Develops two ICs into leads across different teams and shapes the interview loop new PM hires now go through. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Develops product leaders the industry recognizes, and their coaching frameworks outlive their tenure - used by people they never met. Scope: company portfolio and the external craft community.</t>
+          <t>Depth: Develops senior engineers and leaders; builds culture deliberately. Evidenced by: Builds a coaching culture across the product org that other leads' own coaching practice gets measured against. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Develops the next generation of top talent; legacy outlasts tenure. Evidenced by: Develops PMs who go on to lead product organizations elsewhere, and the practice they carry with them traces back to this person's coaching. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -2958,37 +3154,42 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Cagan, *Empowered* (2020); Larson, *Staff Engineer* (2021)</t>
+          <t>Shapes technical direction beyond own work.</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Adopts the team's craft standards fast and flags gaps in them - the missing checklist item, the template that confuses - instead of working around them silently. Scope: their own work meets the bar.</t>
+          <t>Cagan &amp; Jones, EMPOWERED: Ordinary People, Extraordinary Products (Wiley, 2020) — shaping product craft beyond one's own work — what good discovery, specs, and trade-offs look like for other PMs — paired with Larson's Staff-archetype ladder for how that influence scales from one domain to company strategy.</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Contributes reusable craft artifacts - a better interview guide, a sharper spec template - that at least one other PM adopts unprompted. Scope: their team's practice.</t>
+          <t>Depth: Contributes informed opinions in technical discussions. Evidenced by: Offers an informed opinion in a spec review that a more senior PM ultimately weighs alongside their own, without yet being the person others default to. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the local bar by example and review - their discovery notes, specs, and analyses are the ones held up as "this is what good looks like," and their reviews pull others up to it. Scope: a product; the terminal-level craftsperson others calibrate against.</t>
+          <t>Depth: Influences component-level decisions through credibility. Evidenced by: Earns their product area's default trust on discovery-method calls through consistently sound judgment, not because of a title. Scope: a product area.</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Exports practice deliberately across teams - running craft reviews, writing playbooks, and getting discovery or writing standards adopted by teams that don't report anywhere near them. Scope: multiple product areas.</t>
+          <t>Depth: Sets technical direction for a domain; others align to their calls. Evidenced by: Sets the discovery and spec-writing bar their product's team aligns to without being told, handling the hardest ambiguous calls unsupervised. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns the org's product craft agenda - decides which practices to standardize vs. leave local, retires cargo-cult process, and measures whether the bar actually moved. Scope: product org.</t>
+          <t>Depth: Shapes how multiple teams approach problems; trusted tiebreaker. Evidenced by: Becomes the trusted tiebreaker on a craft question that spans three teams' approaches, and the resolution shapes how all three now work. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines product craft beyond the company - published methods, talks, and internal canon that other companies borrow; the company's product reputation is partly their work. Scope: company portfolio and industry.</t>
+          <t>Depth: Influences org-wide technical strategy. Evidenced by: Advises the product org's leadership on craft strategy at organizational scale, influencing standards no single cross-team problem could reach. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Influences company strategic direction through insight. Evidenced by: Shapes the company's strategic direction through craft insight that gets adopted well beyond the product organization. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -3015,37 +3216,42 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Cagan, *Empowered* (2020)</t>
+          <t>Builds the team through hiring and placement.</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Interviews candidates for intern and APM roles with a prepared rubric and writes evidence-based feedback that separates observation from verdict. Scope: interview loops they join.</t>
+          <t>Cagan &amp; Jones, EMPOWERED: Ordinary People, Extraordinary Products (Wiley, 2020) — building the team through hiring and placement is the product leader's compounding lever — a strong PM organization is built one calibrated hire at a time, not backfilled after the fact.</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs strong interviews for PM roles - probes for craft with real-work questions, calibrates scores against the rubric - and their written feedback is specific enough to be decisive in debriefs. Scope: their area's hiring loops.</t>
+          <t>Depth: Participates in interviews; gives clear, evidence-based feedback. Evidenced by: Gives evidence-based interview feedback using the team's existing scorecard, citing the specific answer that drove their rating. Scope: one feature/epic.</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Anchors PM hiring loops - designs interview questions that expose craft rather than polish, spots coached answers, and their hire/no-hire calls hold up over time. Scope: their product's hiring; hiring managers ask for them on close calls.</t>
+          <t>Depth: Runs interviews well; calibrates against a consistent bar. Evidenced by: Runs a PM candidate interview independently and calibrates their rating against the team's existing bar without a debrief coach in the room. Scope: a product area.</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Calibrates the PM interview bar across teams - trains interviewers, audits question quality, and reworks loops that pass confident performers and fail quiet builders. Scope: multiple product areas' hiring.</t>
+          <t>Depth: Shapes hiring for a team; designs loops; makes sound staffing calls. Evidenced by: Designs a new interview loop stage that catches a judgment gap the old loop was missing, and makes the staffing call on a contested hire. Scope: a product/capability (terminal level).</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs the org's PM hiring system - competency-based loops, debrief norms, onboarding handoff - and the org's hiring quality is visibly their work. Scope: product org.</t>
+          <t>Depth: Drives hiring strategy across teams; builds the interviewing bar. Evidenced by: Builds the PM interviewing bar three other teams now hire against, driving hiring strategy across the group. Scope: multiple product areas.</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the company's bar for product talent - the hiring philosophy and craft standards that shape who the company hires and attracts, cited by candidates as why they joined. Scope: company portfolio.</t>
+          <t>Depth: Sets the org's talent strategy. Evidenced by: Sets the product org's talent strategy — leveling, sourcing priorities, workforce plan — for the year. Scope: product organization.</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes company-wide talent philosophy. Evidenced by: Shapes the company's talent philosophy for product roles in a way that outlasts their own tenure in the org. Scope: company portfolio.</t>
         </is>
       </c>
     </row>
@@ -5021,249 +5227,796 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sources</t>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Grounds</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Bland, David &amp; Osterwalder, Alexander. *Testing Business Ideas* (2019).</t>
+          <t>Weekly-touchpoint discovery cadence and the opportunity-solution-tree method</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Torres, Continuous Discovery Habits: Discover Products that Create Customer Value and Business Value (Product Talk LLC, 2021)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Customer interviewing</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>https://www.producttalk.org/continuous-discovery-habits-book/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Bryar, Colin &amp; Carr, Bill. *Working Backwards* (2021).</t>
+          <t>Canonical goal-directed interaction-design method and pattern catalog</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Cooper, Reimann, Cronin &amp; Noessel, About Face: The Essentials of Interaction Design, 4th Edition (Wiley, 2014)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Customer segmentation &amp; personas</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wiley.com/en-us/About+Face%3A+The+Essentials+of+Interaction+Design%2C+4th+Edition-p-9781118766576</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Cagan, Marty. *Inspired: How to Create Tech Products Customers Love*, 2nd ed. (2018), and SVPG writing (svpg.com).</t>
+          <t>Org-level product strategy vs. output-shipping; grounds strategic/commercial leveling</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Perri, Escaping the Build Trap: How Effective Product Management Creates Real Value (O'Reilly, 2018)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Problem statements &amp; outcome framing</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oreilly.com/library/view/escaping-the-build/9781491973783/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Cagan, Marty. *Empowered: Ordinary People, Extraordinary Products* (2020).</t>
+          <t>Jobs-to-be-done theory: circumstance, progress sought, competing alternatives including non-consumption</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Christensen, Hall, Dillon &amp; Duncan, Competing Against Luck: The Story of Innovation and Customer Choice (HarperBusiness, 2016)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Jobs-to-be-done framing</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/competingagainst0000chri</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Christensen, Clayton. *The Innovator's Dilemma* (1997).</t>
+          <t>Assumptions mapping (desirability/viability/feasibility ranked by importance x evidence) and the experiment library</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Bland &amp; Osterwalder, Testing Business Ideas: A Field Guide for Rapid Experimentation (Wiley, 2019)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Assumption mapping &amp; risk framing</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wiley.com/en-us/Testing+Business+Ideas%3A+A+Field+Guide+for+Rapid+Experimentation-p-9781119551447</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Christensen, Clayton; Hall, Taddy; Dillon, Karen; Duncan, David. "Know Your Customers' 'Jobs to Be Done'," *Harvard Business Review* (2016); *Competing Against Luck* (2016).</t>
+          <t>Build-measure-learn loop and validated learning as falsifiable, staged commitment</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Ries, The Lean Startup: How Today's Entrepreneurs Use Continuous Innovation to Create Radically Successful Businesses (Crown Business, 2011)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Assumption testing &amp; experiments</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>https://theleanstartup.com/book</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Cooper, Alan. *The Inmates Are Running the Asylum* (1999).</t>
+          <t>Strategy kernel (diagnosis, guiding policy, coherent action) as the test for real vs. bad strategy</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Rumelt, Good Strategy Bad Strategy: The Difference and Why It Matters (Crown Business, 2011)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Product strategy formulation</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.penguinrandomhouse.com/books/198888/good-strategy-bad-strategy-by-richard-p-rumelt/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Croll, Alistair &amp; Yoskovitz, Benjamin. *Lean Analytics* (2013).</t>
+          <t>Positioning canvas: competitive alternatives, differentiated value, target market characteristics</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Dunford, Obviously Awesome: How to Nail Product Positioning (Ambient Press, 2019)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Positioning &amp; differentiation</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.aprildunford.com/obviously-awesome</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Doerr, John. *Measure What Matters* (2018).</t>
+          <t>SVPG discovery-risk framework (value/usability/feasibility/viability); PM domain-expertise and discovery-judgment anchor</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Cagan, INSPIRED: How to Create Tech Products Customers Love, 2nd Edition (Wiley, 2018)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Product vision narrative</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.svpg.com/inspired-2nd-edition/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Duke, Annie. *Thinking in Bets* (2018).</t>
+          <t>OKR format (objective plus measurable key results) and cascading goal alignment</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Doerr, Measure What Matters (Portfolio/Penguin, 2018)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Goal setting &amp; OKRs</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.whatmatters.com/the-book</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Dunford, April. *Obviously Awesome* (2019).</t>
+          <t>One Metric That Matters, stage-based metrics model, and vanity-metric diagnosis</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Croll &amp; Yoskovitz, Lean Analytics: Use Data to Build a Better Startup Faster (O'Reilly, 2013)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Success metrics &amp; KPI design</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>https://leananalyticsbook.com/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Edmondson, Amy. *The Fearless Organization* (2018).</t>
+          <t>Canonical reference on rigorous online experimentation, confounds and guardrails</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Kohavi, Tang &amp; Xu, Trustworthy Online Controlled Experiments: A Practical Guide to A/B Testing (Cambridge University Press, 2020)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>A/B test design &amp; analysis</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>https://experimentguide.com/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Kahneman, Daniel. *Thinking, Fast and Slow* (2011).</t>
+          <t>System 1 / System 2 reasoning; basis for structured decision-making under uncertainty</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Kahneman, Thinking, Fast and Slow (Farrar, Straus and Giroux, 2011)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Decision quality under uncertainty</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Thinking,_Fast_and_Slow</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Kohavi, Ron; Tang, Diane; Xu, Ya. *Trustworthy Online Controlled Experiments* (2020).</t>
-        </is>
-      </c>
+          <t>Cost-of-delay and queueing-theory economics for prioritization decisions; verified via web search</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Reinertsen, The Principles of Product Development Flow: Second Generation Lean Product Development (Celeritas, 2009)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Prioritization &amp; sequencing</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Larson, Will. *Staff Engineer: Leadership Beyond the Management Track* (2021).</t>
+          <t>Executive trust-building and organizational product-leadership practice</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Cagan &amp; Jones, EMPOWERED: Ordinary People, Extraordinary Products (Wiley, 2020)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Product trio partnership</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.svpg.com/empowered/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Lombardo, C. Todd; McCarthy, Bruce; Ryan, Evan; Connors, Michael. *Product Roadmaps Relaunched* (2017).</t>
+          <t>Requirements elicitation and business-analysis competency standard</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>IIBA, A Guide to the Business Analysis Body of Knowledge (BABOK Guide), Version 3 (2015)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Requirements, specs &amp; acceptance criteria</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.iiba.org/contentassets/a566a72f87314878bbed046681829fb8/business-analysis-body-of-knowledge-babok-guide-v3.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>McClure, Dave. "Startup Metrics for Pirates" (AARRR framework, 2007).</t>
+          <t>Slicing and sequencing work for incremental value delivery</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Patton, User Story Mapping: Discover the Whole Story, Build the Right Product (O'Reilly, 2014)</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Backlog &amp; delivery flow</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oreilly.com/library/view/user-story-mapping/9781491904893/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>McKeown, Greg. *Essentialism* (2014).</t>
+          <t>Business Model Canvas as the standard business-modeling template</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Osterwalder &amp; Pigneur, Business Model Generation (Wiley, 2010)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Business model &amp; unit economics</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>https://www.strategyzer.com/library/business-model-generation</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Minto, Barbara. *The Pyramid Principle* (1987).</t>
+          <t>Value-based pricing and the value cascade, as against cost-plus defaults</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Nagle, Muller &amp; Gruyaert, The Strategy and Tactics of Pricing: A Guide to Growing More Profitably, 7th Edition (Routledge, 2023)</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Pricing &amp; packaging</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>https://www.routledge.com/The-Strategy-and-Tactics-of-Pricing-A-Guide-to-Growing-More-Profitably/Nagle-Muller-Gruyaert/p/book/9781032016825</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Moore, Geoffrey. *Crossing the Chasm*, 3rd ed. (2014).</t>
+          <t>Technology adoption lifecycle and the chasm between early and mainstream markets; whitespace and launch-beachhead strategy</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Moore, Crossing the Chasm: Marketing and Selling High-Tech Products to Mainstream Customers, 3rd Edition (HarperBusiness, 2014; orig. 1991)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Competitive &amp; market analysis</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/crossingthechasm_202002</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Olsen, Dan. *The Lean Product Playbook* (2015).</t>
+          <t>Classic clarity-in-writing reference; grounds written communication leveling</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Zinsser, On Writing Well: The Classic Guide to Writing Nonfiction, 30th Anniversary Edition (Harper Perennial, 2006)</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Product narratives &amp; written communication</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>https://openlibrary.org/books/OL3430145M/On_Writing_Well</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Osterwalder, Alexander &amp; Pigneur, Yves. *Business Model Generation* (2010).</t>
+          <t>Answer-first, structured argument method; grounds executive-communication and design-doc leveling</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Minto, The Minto Pyramid Principle: Logic in Writing, Thinking, and Problem Solving (Minto International, 1996)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Executive communication</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.barbaraminto.com/</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Patton, Jeff. *User Story Mapping* (2014).</t>
-        </is>
-      </c>
+      <c r="A24" s="4" t="inlineStr"/>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Torres, Continuous Discovery Habits: Discover Products that Create Customer Value and Business Value (Product Talk LLC, 2021) — https://www.producttalk.org/continuous-discovery-habits-book/</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr"/>
+      <c r="D24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Perri, Melissa. *Escaping the Build Trap* (2018).</t>
-        </is>
-      </c>
+      <c r="A25" s="4" t="inlineStr"/>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Fitzpatrick, The Mom Test: How to Talk to Customers and Learn If Your Business Is a Good Idea When Everyone Is Lying to You (self-published, 2013) — https://www.momtestbook.com/</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Portigal, Steve. *Interviewing Users* (2013).</t>
-        </is>
-      </c>
+      <c r="A26" s="4" t="inlineStr"/>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>SFIA Foundation, Skills Framework for the Information Age, version 9 (2024) — https://sfia-online.org/en/sfia-9</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr"/>
+      <c r="D26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Ramanujam, Madhavan &amp; Tacke, Georg. *Monetizing Innovation* (2016).</t>
-        </is>
-      </c>
+      <c r="A27" s="4" t="inlineStr"/>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Larson, Staff Engineer: Leadership Beyond the Management Track (self-published, 2021) — https://staffeng.com/book/</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr"/>
+      <c r="D27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>Reinertsen, Donald. *The Principles of Product Development Flow* (2009).</t>
-        </is>
-      </c>
+      <c r="A28" s="4" t="inlineStr"/>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Cagan, INSPIRED: How to Create Tech Products Customers Love, 2nd Edition (Wiley, 2018) — https://www.svpg.com/inspired-2nd-edition/</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr"/>
+      <c r="D28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Ries, Eric. *The Lean Startup* (2011).</t>
-        </is>
-      </c>
+      <c r="A29" s="4" t="inlineStr"/>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Cooper, Reimann, Cronin &amp; Noessel, About Face: The Essentials of Interaction Design, 4th Edition (Wiley, 2014) — https://www.wiley.com/en-us/About+Face%3A+The+Essentials+of+Interaction+Design%2C+4th+Edition-p-9781118766576</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr"/>
+      <c r="D29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>Rumelt, Richard. *Good Strategy Bad Strategy* (2011).</t>
-        </is>
-      </c>
+      <c r="A30" s="4" t="inlineStr"/>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Moore, Crossing the Chasm: Marketing and Selling High-Tech Products to Mainstream Customers, 3rd Edition (HarperBusiness, 2014; orig. 1991) — https://archive.org/details/crossingthechasm_202002</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr"/>
+      <c r="D30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Singer, Ryan. *Shape Up* (Basecamp, 2019).</t>
-        </is>
-      </c>
+      <c r="A31" s="4" t="inlineStr"/>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Perri, Escaping the Build Trap: How Effective Product Management Creates Real Value (O'Reilly, 2018) — https://www.oreilly.com/library/view/escaping-the-build/9781491973783/</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr"/>
+      <c r="D31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Torres, Teresa. *Continuous Discovery Habits* (2021).</t>
-        </is>
-      </c>
+      <c r="A32" s="4" t="inlineStr"/>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Christensen, Hall, Dillon &amp; Duncan, Competing Against Luck: The Story of Innovation and Customer Choice (HarperBusiness, 2016) — https://archive.org/details/competingagainst0000chri</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr"/>
+      <c r="D32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>Muller, Markus. "Decoding Product Management - A Skill Matrix" (Medium, 2023) - trusted fifth source; competency territory only, prose rewritten.</t>
-        </is>
-      </c>
+      <c r="A33" s="4" t="inlineStr"/>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Bland &amp; Osterwalder, Testing Business Ideas: A Field Guide for Rapid Experimentation (Wiley, 2019) — https://www.wiley.com/en-us/Testing+Business+Ideas%3A+A+Field+Guide+for+Rapid+Experimentation-p-9781119551447</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr"/>
+      <c r="D33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Real APM -&gt; Principal PM job postings - seniority and scope calibration cross-check (via the source runs).</t>
-        </is>
-      </c>
+      <c r="A34" s="4" t="inlineStr"/>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Ries, The Lean Startup: How Today's Entrepreneurs Use Continuous Innovation to Create Radically Successful Businesses (Crown Business, 2011) — https://theleanstartup.com/book</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr"/>
+      <c r="D34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr"/>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Rumelt, Good Strategy Bad Strategy: The Difference and Why It Matters (Crown Business, 2011) — https://www.penguinrandomhouse.com/books/198888/good-strategy-bad-strategy-by-richard-p-rumelt/</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr"/>
+      <c r="D35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr"/>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Dunford, Obviously Awesome: How to Nail Product Positioning (Ambient Press, 2019) — https://www.aprildunford.com/obviously-awesome</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr"/>
+      <c r="D36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr"/>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Lombardo, McCarthy, Ryan &amp; Connors, Product Roadmaps Relaunched: How to Set Direction while Embracing Uncertainty (O'Reilly, 2017) — https://www.oreilly.com/library/view/product-roadmaps-relaunched/9781491971710/</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr"/>
+      <c r="D37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr"/>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Doerr, Measure What Matters (Portfolio/Penguin, 2018) — https://www.whatmatters.com/the-book</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr"/>
+      <c r="D38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr"/>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Croll &amp; Yoskovitz, Lean Analytics: Use Data to Build a Better Startup Faster (O'Reilly, 2013) — https://leananalyticsbook.com/</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr"/>
+      <c r="D39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr"/>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Kohavi, Tang &amp; Xu, Trustworthy Online Controlled Experiments: A Practical Guide to A/B Testing (Cambridge University Press, 2020) — https://experimentguide.com/</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr"/>
+      <c r="D40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr"/>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Kahneman, Thinking, Fast and Slow (Farrar, Straus and Giroux, 2011) — https://en.wikipedia.org/wiki/Thinking,_Fast_and_Slow</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr"/>
+      <c r="D41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr"/>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Reinertsen, The Principles of Product Development Flow: Second Generation Lean Product Development (Celeritas, 2009)</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr"/>
+      <c r="D42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr"/>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Cagan &amp; Jones, EMPOWERED: Ordinary People, Extraordinary Products (Wiley, 2020) — https://www.svpg.com/empowered/</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr"/>
+      <c r="D43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr"/>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>IIBA, A Guide to the Business Analysis Body of Knowledge (BABOK Guide), Version 3 (2015) — https://www.iiba.org/contentassets/a566a72f87314878bbed046681829fb8/business-analysis-body-of-knowledge-babok-guide-v3.pdf</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr"/>
+      <c r="D44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr"/>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>ISO/IEC/IEEE, Systems and Software Engineering -- Life Cycle Processes -- Requirements Engineering, ISO/IEC/IEEE 29148:2018 — https://www.iso.org/standard/72089.html</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr"/>
+      <c r="D45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr"/>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Patton, User Story Mapping: Discover the Whole Story, Build the Right Product (O'Reilly, 2014) — https://www.oreilly.com/library/view/user-story-mapping/9781491904893/</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr"/>
+      <c r="D46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr"/>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Osterwalder &amp; Pigneur, Business Model Generation (Wiley, 2010) — https://www.strategyzer.com/library/business-model-generation</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr"/>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Nagle, Muller &amp; Gruyaert, The Strategy and Tactics of Pricing: A Guide to Growing More Profitably, 7th Edition (Routledge, 2023) — https://www.routledge.com/The-Strategy-and-Tactics-of-Pricing-A-Guide-to-Growing-More-Profitably/Nagle-Muller-Gruyaert/p/book/9781032016825</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr"/>
+      <c r="D48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr"/>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Zinsser, On Writing Well: The Classic Guide to Writing Nonfiction, 30th Anniversary Edition (Harper Perennial, 2006) — https://openlibrary.org/books/OL3430145M/On_Writing_Well</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr"/>
+      <c r="D49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr"/>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Minto, The Minto Pyramid Principle: Logic in Writing, Thinking, and Problem Solving (Minto International, 1996) — https://www.barbaraminto.com/</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr"/>
+      <c r="D50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr"/>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Grove, High Output Management (Random House, 1983) — https://www.penguinrandomhouse.com/books/163289/high-output-management-by-andrew-s-grove/</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr"/>
+      <c r="D51" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>